<commit_message>
feat: expand mode one with codex and second stage
</commit_message>
<xml_diff>
--- a/content/game_config.xlsx
+++ b/content/game_config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R39668855b1a44976"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="R7d6ed8e61cff4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="R3ff93fd9d6204a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="R211da2b90ba8498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0f19b35c053c4e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="Rba176a456de746b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="Rdcf4b268ff714642"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="R2ccc5f79707d4f62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13007,22 +13007,48 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="12"/>
-      <x:c r="B25" s="14"/>
-      <x:c r="C25" s="14"/>
-      <x:c r="D25" s="14"/>
-      <x:c r="E25" s="14"/>
+    <x:row r="25" ht="45" customHeight="1">
+      <x:c r="A25" s="12" t="str">
+        <x:v>menu_background</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="n">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="n">
+        <x:v>720</x:v>
+      </x:c>
       <x:c r="F25" s="12"/>
-      <x:c r="G25" s="12"/>
+      <x:c r="G25" s="12" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
       <x:c r="H25" s="13"/>
-      <x:c r="I25" s="14"/>
-      <x:c r="J25" s="14"/>
-      <x:c r="K25" s="14"/>
-      <x:c r="L25" s="14"/>
-      <x:c r="M25" s="14"/>
-      <x:c r="N25" s="13"/>
-      <x:c r="O25" s="14"/>
+      <x:c r="I25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M25" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N25" s="13" t="str">
+        <x:v>开始、暂停和结算菜单背景；先在图片资源登记素材名</x:v>
+      </x:c>
+      <x:c r="O25" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="12"/>
@@ -15218,7 +15244,7 @@
       <x:c r="O154" s="14"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="6">
     <x:dataValidation type="list" sqref="G5:G154">
       <x:formula1>"ninepatch,stretch,keep"</x:formula1>
     </x:dataValidation>
@@ -15231,6 +15257,12 @@
     <x:dataValidation type="list" sqref="O24">
       <x:formula1>"0,1"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="G25">
+      <x:formula1>"ninepatch,stretch,keep"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="O25">
+      <x:formula1>"0,1"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: add persistent unlocks and squad selection
</commit_message>
<xml_diff>
--- a/content/game_config.xlsx
+++ b/content/game_config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0f19b35c053c4e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="Rba176a456de746b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="Rdcf4b268ff714642"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="R2ccc5f79707d4f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R5a6efd7a93fb4985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="R1ac26bf8e5574af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="R274f2f6833b64486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="R63a0c9a1e0664d86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,8 +53,25 @@
       <x:color rgb="FF263443"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF2A2024"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF7D2436"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2A2024"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,19 +88,86 @@
         <x:fgColor rgb="FFFFF8DE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
         <x:color rgb="FFBCC8D0"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5B45A"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -129,6 +213,107 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -521,6 +706,22 @@
         <x:v>在图片资源表登记背景后，把资源名填到UI表dialog_background的素材列；stretch铺满，keep保留比例。</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="55" t="str">
+        <x:v>模式一剧情</x:v>
+      </x:c>
+      <x:c r="B25" s="56" t="str">
+        <x:v>段落名可填写mode1_opening、mode1_won、mode1_stage2_opening、mode1_stage3_opening、mode1_final_won、mode1_lost。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="55" t="str">
+        <x:v>编队界面</x:v>
+      </x:c>
+      <x:c r="B26" s="56" t="str">
+        <x:v>UI表的squad_开头控件可修改位置、尺寸、文字和素材；游戏中按F3打开编队。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -534,7 +735,7 @@
     <x:col min="2" max="2" width="12.5" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="7.75" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="65.62999725341797" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="9" hidden="0" customWidth="1"/>
@@ -1623,244 +1824,676 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="12"/>
-      <x:c r="C22" s="14"/>
-      <x:c r="D22" s="12"/>
-      <x:c r="E22" s="13"/>
-      <x:c r="F22" s="12"/>
-      <x:c r="G22" s="12"/>
-      <x:c r="H22" s="14"/>
-      <x:c r="I22" s="14"/>
-      <x:c r="J22" s="15"/>
-      <x:c r="K22" s="14"/>
-      <x:c r="L22" s="12"/>
-      <x:c r="M22" s="12"/>
-      <x:c r="N22" s="14"/>
-      <x:c r="O22" s="14"/>
-      <x:c r="P22" s="15"/>
-      <x:c r="Q22" s="14"/>
-      <x:c r="R22" s="12"/>
+      <x:c r="A22" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B22" s="58" t="str">
+        <x:v>mode1_opening</x:v>
+      </x:c>
+      <x:c r="C22" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E22" s="58" t="str">
+        <x:v>裂隙已经越过警戒线。元素尚未回应我，但剑还在手里。</x:v>
+      </x:c>
+      <x:c r="F22" s="58" t="str">
+        <x:v>saria</x:v>
+      </x:c>
+      <x:c r="G22" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H22" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I22" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J22" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K22" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M22" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N22" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O22" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P22" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q22" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R22" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="12"/>
-      <x:c r="C23" s="14"/>
-      <x:c r="D23" s="12"/>
-      <x:c r="E23" s="13"/>
-      <x:c r="F23" s="12"/>
-      <x:c r="G23" s="12"/>
-      <x:c r="H23" s="14"/>
-      <x:c r="I23" s="14"/>
-      <x:c r="J23" s="15"/>
-      <x:c r="K23" s="14"/>
-      <x:c r="L23" s="12"/>
-      <x:c r="M23" s="12"/>
-      <x:c r="N23" s="14"/>
-      <x:c r="O23" s="14"/>
-      <x:c r="P23" s="15"/>
-      <x:c r="Q23" s="14"/>
-      <x:c r="R23" s="12"/>
+      <x:c r="A23" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B23" s="58" t="str">
+        <x:v>mode1_opening</x:v>
+      </x:c>
+      <x:c r="C23" s="57" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D23" s="58" t="str">
+        <x:v>通讯员</x:v>
+      </x:c>
+      <x:c r="E23" s="58" t="str">
+        <x:v>水晶会收集敌人的残响。每次升级都能改写攻击方式，弹道与支援也会随构筑增长。</x:v>
+      </x:c>
+      <x:c r="F23" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="G23" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H23" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I23" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J23" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K23" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" s="58" t="str">
+        <x:v>saria</x:v>
+      </x:c>
+      <x:c r="M23" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N23" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O23" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P23" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q23" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R23" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="14"/>
-      <x:c r="B24" s="12"/>
-      <x:c r="C24" s="14"/>
-      <x:c r="D24" s="12"/>
-      <x:c r="E24" s="13"/>
-      <x:c r="F24" s="12"/>
-      <x:c r="G24" s="12"/>
-      <x:c r="H24" s="14"/>
-      <x:c r="I24" s="14"/>
-      <x:c r="J24" s="15"/>
-      <x:c r="K24" s="14"/>
-      <x:c r="L24" s="12"/>
-      <x:c r="M24" s="12"/>
-      <x:c r="N24" s="14"/>
-      <x:c r="O24" s="14"/>
-      <x:c r="P24" s="15"/>
-      <x:c r="Q24" s="14"/>
-      <x:c r="R24" s="12"/>
+      <x:c r="A24" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B24" s="58" t="str">
+        <x:v>mode1_opening</x:v>
+      </x:c>
+      <x:c r="C24" s="57" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D24" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E24" s="58" t="str">
+        <x:v>那就从这里开始。守住五分半，把右侧涌来的东西全部送回去。</x:v>
+      </x:c>
+      <x:c r="F24" s="58" t="str">
+        <x:v>saria-soft</x:v>
+      </x:c>
+      <x:c r="G24" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H24" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I24" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J24" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K24" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M24" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N24" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O24" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P24" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q24" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R24" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="14"/>
-      <x:c r="B25" s="12"/>
-      <x:c r="C25" s="14"/>
-      <x:c r="D25" s="12"/>
-      <x:c r="E25" s="13"/>
-      <x:c r="F25" s="12"/>
-      <x:c r="G25" s="12"/>
-      <x:c r="H25" s="14"/>
-      <x:c r="I25" s="14"/>
-      <x:c r="J25" s="15"/>
-      <x:c r="K25" s="14"/>
-      <x:c r="L25" s="12"/>
-      <x:c r="M25" s="12"/>
-      <x:c r="N25" s="14"/>
-      <x:c r="O25" s="14"/>
-      <x:c r="P25" s="15"/>
-      <x:c r="Q25" s="14"/>
-      <x:c r="R25" s="12"/>
+      <x:c r="A25" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B25" s="58" t="str">
+        <x:v>mode1_won</x:v>
+      </x:c>
+      <x:c r="C25" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E25" s="58" t="str">
+        <x:v>第一道裂隙关闭了。水晶记录下了这次构筑，下一关会有新的同伴回应。</x:v>
+      </x:c>
+      <x:c r="F25" s="58" t="str">
+        <x:v>saria-soft</x:v>
+      </x:c>
+      <x:c r="G25" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H25" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I25" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J25" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K25" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M25" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N25" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O25" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P25" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q25" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R25" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="14"/>
-      <x:c r="B26" s="12"/>
-      <x:c r="C26" s="14"/>
-      <x:c r="D26" s="12"/>
-      <x:c r="E26" s="13"/>
-      <x:c r="F26" s="12"/>
-      <x:c r="G26" s="12"/>
-      <x:c r="H26" s="14"/>
-      <x:c r="I26" s="14"/>
-      <x:c r="J26" s="15"/>
-      <x:c r="K26" s="14"/>
-      <x:c r="L26" s="12"/>
-      <x:c r="M26" s="12"/>
-      <x:c r="N26" s="14"/>
-      <x:c r="O26" s="14"/>
-      <x:c r="P26" s="15"/>
-      <x:c r="Q26" s="14"/>
-      <x:c r="R26" s="12"/>
+      <x:c r="A26" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B26" s="58" t="str">
+        <x:v>mode1_stage2_opening</x:v>
+      </x:c>
+      <x:c r="C26" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="58" t="str">
+        <x:v>宵宫</x:v>
+      </x:c>
+      <x:c r="E26" s="58" t="str">
+        <x:v>通讯接通。第二道裂隙已经变成赤潮，我从高台提供火力。</x:v>
+      </x:c>
+      <x:c r="F26" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="G26" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H26" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I26" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J26" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K26" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="58" t="str">
+        <x:v>saria</x:v>
+      </x:c>
+      <x:c r="M26" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N26" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O26" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P26" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q26" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R26" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="14"/>
-      <x:c r="B27" s="12"/>
-      <x:c r="C27" s="14"/>
-      <x:c r="D27" s="12"/>
-      <x:c r="E27" s="13"/>
-      <x:c r="F27" s="12"/>
-      <x:c r="G27" s="12"/>
-      <x:c r="H27" s="14"/>
-      <x:c r="I27" s="14"/>
-      <x:c r="J27" s="15"/>
-      <x:c r="K27" s="14"/>
-      <x:c r="L27" s="12"/>
-      <x:c r="M27" s="12"/>
-      <x:c r="N27" s="14"/>
-      <x:c r="O27" s="14"/>
-      <x:c r="P27" s="15"/>
-      <x:c r="Q27" s="14"/>
-      <x:c r="R27" s="12"/>
+      <x:c r="A27" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B27" s="58" t="str">
+        <x:v>mode1_stage2_opening</x:v>
+      </x:c>
+      <x:c r="C27" s="57" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D27" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E27" s="58" t="str">
+        <x:v>上一关的强化已经消散，但元素选择和新的构筑会再次回应。两个人守住三条路线。</x:v>
+      </x:c>
+      <x:c r="F27" s="58" t="str">
+        <x:v>saria-soft</x:v>
+      </x:c>
+      <x:c r="G27" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H27" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I27" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J27" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K27" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M27" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N27" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O27" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P27" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q27" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R27" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="14"/>
-      <x:c r="B28" s="12"/>
-      <x:c r="C28" s="14"/>
-      <x:c r="D28" s="12"/>
-      <x:c r="E28" s="13"/>
-      <x:c r="F28" s="12"/>
-      <x:c r="G28" s="12"/>
-      <x:c r="H28" s="14"/>
-      <x:c r="I28" s="14"/>
-      <x:c r="J28" s="15"/>
-      <x:c r="K28" s="14"/>
-      <x:c r="L28" s="12"/>
-      <x:c r="M28" s="12"/>
-      <x:c r="N28" s="14"/>
-      <x:c r="O28" s="14"/>
-      <x:c r="P28" s="15"/>
-      <x:c r="Q28" s="14"/>
-      <x:c r="R28" s="12"/>
+      <x:c r="A28" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B28" s="58" t="str">
+        <x:v>mode1_stage3_opening</x:v>
+      </x:c>
+      <x:c r="C28" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D28" s="58" t="str">
+        <x:v>芙宁娜</x:v>
+      </x:c>
+      <x:c r="E28" s="58" t="str">
+        <x:v>第三道裂隙已经结晶化，路线正在上下错位。水域会替大家维持生命。</x:v>
+      </x:c>
+      <x:c r="F28" s="58" t="str">
+        <x:v>muelsyse</x:v>
+      </x:c>
+      <x:c r="G28" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H28" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I28" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J28" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K28" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M28" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N28" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O28" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P28" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q28" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R28" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="14"/>
-      <x:c r="B29" s="12"/>
-      <x:c r="C29" s="14"/>
-      <x:c r="D29" s="12"/>
-      <x:c r="E29" s="13"/>
-      <x:c r="F29" s="12"/>
-      <x:c r="G29" s="12"/>
-      <x:c r="H29" s="14"/>
-      <x:c r="I29" s="14"/>
-      <x:c r="J29" s="15"/>
-      <x:c r="K29" s="14"/>
-      <x:c r="L29" s="12"/>
-      <x:c r="M29" s="12"/>
-      <x:c r="N29" s="14"/>
-      <x:c r="O29" s="14"/>
-      <x:c r="P29" s="15"/>
-      <x:c r="Q29" s="14"/>
-      <x:c r="R29" s="12"/>
+      <x:c r="A29" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B29" s="58" t="str">
+        <x:v>mode1_stage3_opening</x:v>
+      </x:c>
+      <x:c r="C29" s="57" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D29" s="58" t="str">
+        <x:v>宵宫</x:v>
+      </x:c>
+      <x:c r="E29" s="58" t="str">
+        <x:v>黑曜母巢会周期召来疾行兽，我负责清掉它的护卫。</x:v>
+      </x:c>
+      <x:c r="F29" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="G29" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H29" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I29" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J29" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K29" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="58" t="str">
+        <x:v>muelsyse</x:v>
+      </x:c>
+      <x:c r="M29" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N29" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O29" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P29" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q29" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R29" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="14"/>
-      <x:c r="B30" s="12"/>
-      <x:c r="C30" s="14"/>
-      <x:c r="D30" s="12"/>
-      <x:c r="E30" s="13"/>
-      <x:c r="F30" s="12"/>
-      <x:c r="G30" s="12"/>
-      <x:c r="H30" s="14"/>
-      <x:c r="I30" s="14"/>
-      <x:c r="J30" s="15"/>
-      <x:c r="K30" s="14"/>
-      <x:c r="L30" s="12"/>
-      <x:c r="M30" s="12"/>
-      <x:c r="N30" s="14"/>
-      <x:c r="O30" s="14"/>
-      <x:c r="P30" s="15"/>
-      <x:c r="Q30" s="14"/>
-      <x:c r="R30" s="12"/>
+      <x:c r="A30" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B30" s="58" t="str">
+        <x:v>mode1_stage3_opening</x:v>
+      </x:c>
+      <x:c r="C30" s="57" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D30" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E30" s="58" t="str">
+        <x:v>三人到齐。重新选择元素与构筑，把母巢留在这里。</x:v>
+      </x:c>
+      <x:c r="F30" s="58" t="str">
+        <x:v>saria-soft</x:v>
+      </x:c>
+      <x:c r="G30" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H30" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I30" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J30" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K30" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="58" t="str">
+        <x:v>muelsyse</x:v>
+      </x:c>
+      <x:c r="M30" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N30" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O30" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P30" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q30" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R30" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
-      <x:c r="A31" s="14"/>
-      <x:c r="B31" s="12"/>
-      <x:c r="C31" s="14"/>
-      <x:c r="D31" s="12"/>
-      <x:c r="E31" s="13"/>
-      <x:c r="F31" s="12"/>
-      <x:c r="G31" s="12"/>
-      <x:c r="H31" s="14"/>
-      <x:c r="I31" s="14"/>
-      <x:c r="J31" s="15"/>
-      <x:c r="K31" s="14"/>
-      <x:c r="L31" s="12"/>
-      <x:c r="M31" s="12"/>
-      <x:c r="N31" s="14"/>
-      <x:c r="O31" s="14"/>
-      <x:c r="P31" s="15"/>
-      <x:c r="Q31" s="14"/>
-      <x:c r="R31" s="12"/>
+      <x:c r="A31" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B31" s="58" t="str">
+        <x:v>mode1_final_won</x:v>
+      </x:c>
+      <x:c r="C31" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D31" s="58" t="str">
+        <x:v>芙宁娜</x:v>
+      </x:c>
+      <x:c r="E31" s="58" t="str">
+        <x:v>黑曜母巢停止活动，三道裂隙都已经安静下来。</x:v>
+      </x:c>
+      <x:c r="F31" s="58" t="str">
+        <x:v>muelsyse</x:v>
+      </x:c>
+      <x:c r="G31" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H31" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I31" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J31" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K31" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="58" t="str">
+        <x:v>saria</x:v>
+      </x:c>
+      <x:c r="M31" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N31" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O31" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P31" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q31" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R31" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
-      <x:c r="A32" s="14"/>
-      <x:c r="B32" s="12"/>
-      <x:c r="C32" s="14"/>
-      <x:c r="D32" s="12"/>
-      <x:c r="E32" s="13"/>
-      <x:c r="F32" s="12"/>
-      <x:c r="G32" s="12"/>
-      <x:c r="H32" s="14"/>
-      <x:c r="I32" s="14"/>
-      <x:c r="J32" s="15"/>
-      <x:c r="K32" s="14"/>
-      <x:c r="L32" s="12"/>
-      <x:c r="M32" s="12"/>
-      <x:c r="N32" s="14"/>
-      <x:c r="O32" s="14"/>
-      <x:c r="P32" s="15"/>
-      <x:c r="Q32" s="14"/>
-      <x:c r="R32" s="12"/>
+      <x:c r="A32" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B32" s="58" t="str">
+        <x:v>mode1_final_won</x:v>
+      </x:c>
+      <x:c r="C32" s="57" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D32" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E32" s="58" t="str">
+        <x:v>模式一的防线全部守住，水晶已经记录新的角色与卡牌。</x:v>
+      </x:c>
+      <x:c r="F32" s="58" t="str">
+        <x:v>saria-soft</x:v>
+      </x:c>
+      <x:c r="G32" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H32" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I32" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J32" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K32" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="58" t="str">
+        <x:v>muelsyse</x:v>
+      </x:c>
+      <x:c r="M32" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N32" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O32" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P32" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q32" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R32" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
-      <x:c r="A33" s="14"/>
-      <x:c r="B33" s="12"/>
-      <x:c r="C33" s="14"/>
-      <x:c r="D33" s="12"/>
-      <x:c r="E33" s="13"/>
-      <x:c r="F33" s="12"/>
-      <x:c r="G33" s="12"/>
-      <x:c r="H33" s="14"/>
-      <x:c r="I33" s="14"/>
-      <x:c r="J33" s="15"/>
-      <x:c r="K33" s="14"/>
-      <x:c r="L33" s="12"/>
-      <x:c r="M33" s="12"/>
-      <x:c r="N33" s="14"/>
-      <x:c r="O33" s="14"/>
-      <x:c r="P33" s="15"/>
-      <x:c r="Q33" s="14"/>
-      <x:c r="R33" s="12"/>
+      <x:c r="A33" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B33" s="58" t="str">
+        <x:v>mode1_lost</x:v>
+      </x:c>
+      <x:c r="C33" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D33" s="58" t="str">
+        <x:v>旅行者</x:v>
+      </x:c>
+      <x:c r="E33" s="58" t="str">
+        <x:v>水晶破碎前保住了核心记录。重来一次，这次把弹道铺满整条路线。</x:v>
+      </x:c>
+      <x:c r="F33" s="58" t="str">
+        <x:v>saria</x:v>
+      </x:c>
+      <x:c r="G33" s="58" t="str">
+        <x:v>left</x:v>
+      </x:c>
+      <x:c r="H33" s="57" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I33" s="57" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J33" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K33" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="58" t="str">
+        <x:v>jessica</x:v>
+      </x:c>
+      <x:c r="M33" s="58" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="N33" s="57" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="O33" s="57" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="P33" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q33" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R33" s="58" t="str">
+        <x:v>main</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
       <x:c r="A34" s="14"/>
@@ -11281,6 +11914,1206 @@
       <x:c r="P504" s="15"/>
       <x:c r="Q504" s="14"/>
       <x:c r="R504" s="12"/>
+    </x:row>
+    <x:row r="505">
+      <x:c r="A505" s="23"/>
+      <x:c r="B505" s="24"/>
+      <x:c r="C505" s="24"/>
+      <x:c r="D505" s="24"/>
+      <x:c r="E505" s="24"/>
+      <x:c r="F505" s="24"/>
+      <x:c r="G505" s="24"/>
+      <x:c r="H505" s="24"/>
+      <x:c r="I505" s="24"/>
+      <x:c r="J505" s="24"/>
+      <x:c r="K505" s="24"/>
+      <x:c r="L505" s="24"/>
+      <x:c r="M505" s="24"/>
+      <x:c r="N505" s="24"/>
+      <x:c r="O505" s="24"/>
+      <x:c r="P505" s="24"/>
+      <x:c r="Q505" s="24"/>
+      <x:c r="R505" s="25"/>
+    </x:row>
+    <x:row r="506">
+      <x:c r="A506" s="26"/>
+      <x:c r="B506" s="27"/>
+      <x:c r="C506" s="27"/>
+      <x:c r="D506" s="27"/>
+      <x:c r="E506" s="27"/>
+      <x:c r="F506" s="27"/>
+      <x:c r="G506" s="27"/>
+      <x:c r="H506" s="27"/>
+      <x:c r="I506" s="27"/>
+      <x:c r="J506" s="27"/>
+      <x:c r="K506" s="27"/>
+      <x:c r="L506" s="27"/>
+      <x:c r="M506" s="27"/>
+      <x:c r="N506" s="27"/>
+      <x:c r="O506" s="27"/>
+      <x:c r="P506" s="27"/>
+      <x:c r="Q506" s="27"/>
+      <x:c r="R506" s="28"/>
+    </x:row>
+    <x:row r="507">
+      <x:c r="A507" s="26"/>
+      <x:c r="B507" s="27"/>
+      <x:c r="C507" s="27"/>
+      <x:c r="D507" s="27"/>
+      <x:c r="E507" s="27"/>
+      <x:c r="F507" s="27"/>
+      <x:c r="G507" s="27"/>
+      <x:c r="H507" s="27"/>
+      <x:c r="I507" s="27"/>
+      <x:c r="J507" s="27"/>
+      <x:c r="K507" s="27"/>
+      <x:c r="L507" s="27"/>
+      <x:c r="M507" s="27"/>
+      <x:c r="N507" s="27"/>
+      <x:c r="O507" s="27"/>
+      <x:c r="P507" s="27"/>
+      <x:c r="Q507" s="27"/>
+      <x:c r="R507" s="28"/>
+    </x:row>
+    <x:row r="508">
+      <x:c r="A508" s="26"/>
+      <x:c r="B508" s="27"/>
+      <x:c r="C508" s="27"/>
+      <x:c r="D508" s="27"/>
+      <x:c r="E508" s="27"/>
+      <x:c r="F508" s="27"/>
+      <x:c r="G508" s="27"/>
+      <x:c r="H508" s="27"/>
+      <x:c r="I508" s="27"/>
+      <x:c r="J508" s="27"/>
+      <x:c r="K508" s="27"/>
+      <x:c r="L508" s="27"/>
+      <x:c r="M508" s="27"/>
+      <x:c r="N508" s="27"/>
+      <x:c r="O508" s="27"/>
+      <x:c r="P508" s="27"/>
+      <x:c r="Q508" s="27"/>
+      <x:c r="R508" s="28"/>
+    </x:row>
+    <x:row r="509">
+      <x:c r="A509" s="26"/>
+      <x:c r="B509" s="27"/>
+      <x:c r="C509" s="27"/>
+      <x:c r="D509" s="27"/>
+      <x:c r="E509" s="27"/>
+      <x:c r="F509" s="27"/>
+      <x:c r="G509" s="27"/>
+      <x:c r="H509" s="27"/>
+      <x:c r="I509" s="27"/>
+      <x:c r="J509" s="27"/>
+      <x:c r="K509" s="27"/>
+      <x:c r="L509" s="27"/>
+      <x:c r="M509" s="27"/>
+      <x:c r="N509" s="27"/>
+      <x:c r="O509" s="27"/>
+      <x:c r="P509" s="27"/>
+      <x:c r="Q509" s="27"/>
+      <x:c r="R509" s="28"/>
+    </x:row>
+    <x:row r="510">
+      <x:c r="A510" s="26"/>
+      <x:c r="B510" s="27"/>
+      <x:c r="C510" s="27"/>
+      <x:c r="D510" s="27"/>
+      <x:c r="E510" s="27"/>
+      <x:c r="F510" s="27"/>
+      <x:c r="G510" s="27"/>
+      <x:c r="H510" s="27"/>
+      <x:c r="I510" s="27"/>
+      <x:c r="J510" s="27"/>
+      <x:c r="K510" s="27"/>
+      <x:c r="L510" s="27"/>
+      <x:c r="M510" s="27"/>
+      <x:c r="N510" s="27"/>
+      <x:c r="O510" s="27"/>
+      <x:c r="P510" s="27"/>
+      <x:c r="Q510" s="27"/>
+      <x:c r="R510" s="28"/>
+    </x:row>
+    <x:row r="511">
+      <x:c r="A511" s="26"/>
+      <x:c r="B511" s="27"/>
+      <x:c r="C511" s="27"/>
+      <x:c r="D511" s="27"/>
+      <x:c r="E511" s="27"/>
+      <x:c r="F511" s="27"/>
+      <x:c r="G511" s="27"/>
+      <x:c r="H511" s="27"/>
+      <x:c r="I511" s="27"/>
+      <x:c r="J511" s="27"/>
+      <x:c r="K511" s="27"/>
+      <x:c r="L511" s="27"/>
+      <x:c r="M511" s="27"/>
+      <x:c r="N511" s="27"/>
+      <x:c r="O511" s="27"/>
+      <x:c r="P511" s="27"/>
+      <x:c r="Q511" s="27"/>
+      <x:c r="R511" s="28"/>
+    </x:row>
+    <x:row r="512">
+      <x:c r="A512" s="26"/>
+      <x:c r="B512" s="27"/>
+      <x:c r="C512" s="27"/>
+      <x:c r="D512" s="27"/>
+      <x:c r="E512" s="27"/>
+      <x:c r="F512" s="27"/>
+      <x:c r="G512" s="27"/>
+      <x:c r="H512" s="27"/>
+      <x:c r="I512" s="27"/>
+      <x:c r="J512" s="27"/>
+      <x:c r="K512" s="27"/>
+      <x:c r="L512" s="27"/>
+      <x:c r="M512" s="27"/>
+      <x:c r="N512" s="27"/>
+      <x:c r="O512" s="27"/>
+      <x:c r="P512" s="27"/>
+      <x:c r="Q512" s="27"/>
+      <x:c r="R512" s="28"/>
+    </x:row>
+    <x:row r="513">
+      <x:c r="A513" s="26"/>
+      <x:c r="B513" s="27"/>
+      <x:c r="C513" s="27"/>
+      <x:c r="D513" s="27"/>
+      <x:c r="E513" s="27"/>
+      <x:c r="F513" s="27"/>
+      <x:c r="G513" s="27"/>
+      <x:c r="H513" s="27"/>
+      <x:c r="I513" s="27"/>
+      <x:c r="J513" s="27"/>
+      <x:c r="K513" s="27"/>
+      <x:c r="L513" s="27"/>
+      <x:c r="M513" s="27"/>
+      <x:c r="N513" s="27"/>
+      <x:c r="O513" s="27"/>
+      <x:c r="P513" s="27"/>
+      <x:c r="Q513" s="27"/>
+      <x:c r="R513" s="28"/>
+    </x:row>
+    <x:row r="514">
+      <x:c r="A514" s="26"/>
+      <x:c r="B514" s="27"/>
+      <x:c r="C514" s="27"/>
+      <x:c r="D514" s="27"/>
+      <x:c r="E514" s="27"/>
+      <x:c r="F514" s="27"/>
+      <x:c r="G514" s="27"/>
+      <x:c r="H514" s="27"/>
+      <x:c r="I514" s="27"/>
+      <x:c r="J514" s="27"/>
+      <x:c r="K514" s="27"/>
+      <x:c r="L514" s="27"/>
+      <x:c r="M514" s="27"/>
+      <x:c r="N514" s="27"/>
+      <x:c r="O514" s="27"/>
+      <x:c r="P514" s="27"/>
+      <x:c r="Q514" s="27"/>
+      <x:c r="R514" s="28"/>
+    </x:row>
+    <x:row r="515">
+      <x:c r="A515" s="26"/>
+      <x:c r="B515" s="27"/>
+      <x:c r="C515" s="27"/>
+      <x:c r="D515" s="27"/>
+      <x:c r="E515" s="27"/>
+      <x:c r="F515" s="27"/>
+      <x:c r="G515" s="27"/>
+      <x:c r="H515" s="27"/>
+      <x:c r="I515" s="27"/>
+      <x:c r="J515" s="27"/>
+      <x:c r="K515" s="27"/>
+      <x:c r="L515" s="27"/>
+      <x:c r="M515" s="27"/>
+      <x:c r="N515" s="27"/>
+      <x:c r="O515" s="27"/>
+      <x:c r="P515" s="27"/>
+      <x:c r="Q515" s="27"/>
+      <x:c r="R515" s="28"/>
+    </x:row>
+    <x:row r="516">
+      <x:c r="A516" s="26"/>
+      <x:c r="B516" s="27"/>
+      <x:c r="C516" s="27"/>
+      <x:c r="D516" s="27"/>
+      <x:c r="E516" s="27"/>
+      <x:c r="F516" s="27"/>
+      <x:c r="G516" s="27"/>
+      <x:c r="H516" s="27"/>
+      <x:c r="I516" s="27"/>
+      <x:c r="J516" s="27"/>
+      <x:c r="K516" s="27"/>
+      <x:c r="L516" s="27"/>
+      <x:c r="M516" s="27"/>
+      <x:c r="N516" s="27"/>
+      <x:c r="O516" s="27"/>
+      <x:c r="P516" s="27"/>
+      <x:c r="Q516" s="27"/>
+      <x:c r="R516" s="28"/>
+    </x:row>
+    <x:row r="517">
+      <x:c r="A517" s="26"/>
+      <x:c r="B517" s="27"/>
+      <x:c r="C517" s="27"/>
+      <x:c r="D517" s="27"/>
+      <x:c r="E517" s="27"/>
+      <x:c r="F517" s="27"/>
+      <x:c r="G517" s="27"/>
+      <x:c r="H517" s="27"/>
+      <x:c r="I517" s="27"/>
+      <x:c r="J517" s="27"/>
+      <x:c r="K517" s="27"/>
+      <x:c r="L517" s="27"/>
+      <x:c r="M517" s="27"/>
+      <x:c r="N517" s="27"/>
+      <x:c r="O517" s="27"/>
+      <x:c r="P517" s="27"/>
+      <x:c r="Q517" s="27"/>
+      <x:c r="R517" s="28"/>
+    </x:row>
+    <x:row r="518">
+      <x:c r="A518" s="26"/>
+      <x:c r="B518" s="27"/>
+      <x:c r="C518" s="27"/>
+      <x:c r="D518" s="27"/>
+      <x:c r="E518" s="27"/>
+      <x:c r="F518" s="27"/>
+      <x:c r="G518" s="27"/>
+      <x:c r="H518" s="27"/>
+      <x:c r="I518" s="27"/>
+      <x:c r="J518" s="27"/>
+      <x:c r="K518" s="27"/>
+      <x:c r="L518" s="27"/>
+      <x:c r="M518" s="27"/>
+      <x:c r="N518" s="27"/>
+      <x:c r="O518" s="27"/>
+      <x:c r="P518" s="27"/>
+      <x:c r="Q518" s="27"/>
+      <x:c r="R518" s="28"/>
+    </x:row>
+    <x:row r="519">
+      <x:c r="A519" s="26"/>
+      <x:c r="B519" s="27"/>
+      <x:c r="C519" s="27"/>
+      <x:c r="D519" s="27"/>
+      <x:c r="E519" s="27"/>
+      <x:c r="F519" s="27"/>
+      <x:c r="G519" s="27"/>
+      <x:c r="H519" s="27"/>
+      <x:c r="I519" s="27"/>
+      <x:c r="J519" s="27"/>
+      <x:c r="K519" s="27"/>
+      <x:c r="L519" s="27"/>
+      <x:c r="M519" s="27"/>
+      <x:c r="N519" s="27"/>
+      <x:c r="O519" s="27"/>
+      <x:c r="P519" s="27"/>
+      <x:c r="Q519" s="27"/>
+      <x:c r="R519" s="28"/>
+    </x:row>
+    <x:row r="520">
+      <x:c r="A520" s="26"/>
+      <x:c r="B520" s="27"/>
+      <x:c r="C520" s="27"/>
+      <x:c r="D520" s="27"/>
+      <x:c r="E520" s="27"/>
+      <x:c r="F520" s="27"/>
+      <x:c r="G520" s="27"/>
+      <x:c r="H520" s="27"/>
+      <x:c r="I520" s="27"/>
+      <x:c r="J520" s="27"/>
+      <x:c r="K520" s="27"/>
+      <x:c r="L520" s="27"/>
+      <x:c r="M520" s="27"/>
+      <x:c r="N520" s="27"/>
+      <x:c r="O520" s="27"/>
+      <x:c r="P520" s="27"/>
+      <x:c r="Q520" s="27"/>
+      <x:c r="R520" s="28"/>
+    </x:row>
+    <x:row r="521">
+      <x:c r="A521" s="26"/>
+      <x:c r="B521" s="27"/>
+      <x:c r="C521" s="27"/>
+      <x:c r="D521" s="27"/>
+      <x:c r="E521" s="27"/>
+      <x:c r="F521" s="27"/>
+      <x:c r="G521" s="27"/>
+      <x:c r="H521" s="27"/>
+      <x:c r="I521" s="27"/>
+      <x:c r="J521" s="27"/>
+      <x:c r="K521" s="27"/>
+      <x:c r="L521" s="27"/>
+      <x:c r="M521" s="27"/>
+      <x:c r="N521" s="27"/>
+      <x:c r="O521" s="27"/>
+      <x:c r="P521" s="27"/>
+      <x:c r="Q521" s="27"/>
+      <x:c r="R521" s="28"/>
+    </x:row>
+    <x:row r="522">
+      <x:c r="A522" s="26"/>
+      <x:c r="B522" s="27"/>
+      <x:c r="C522" s="27"/>
+      <x:c r="D522" s="27"/>
+      <x:c r="E522" s="27"/>
+      <x:c r="F522" s="27"/>
+      <x:c r="G522" s="27"/>
+      <x:c r="H522" s="27"/>
+      <x:c r="I522" s="27"/>
+      <x:c r="J522" s="27"/>
+      <x:c r="K522" s="27"/>
+      <x:c r="L522" s="27"/>
+      <x:c r="M522" s="27"/>
+      <x:c r="N522" s="27"/>
+      <x:c r="O522" s="27"/>
+      <x:c r="P522" s="27"/>
+      <x:c r="Q522" s="27"/>
+      <x:c r="R522" s="28"/>
+    </x:row>
+    <x:row r="523">
+      <x:c r="A523" s="26"/>
+      <x:c r="B523" s="27"/>
+      <x:c r="C523" s="27"/>
+      <x:c r="D523" s="27"/>
+      <x:c r="E523" s="27"/>
+      <x:c r="F523" s="27"/>
+      <x:c r="G523" s="27"/>
+      <x:c r="H523" s="27"/>
+      <x:c r="I523" s="27"/>
+      <x:c r="J523" s="27"/>
+      <x:c r="K523" s="27"/>
+      <x:c r="L523" s="27"/>
+      <x:c r="M523" s="27"/>
+      <x:c r="N523" s="27"/>
+      <x:c r="O523" s="27"/>
+      <x:c r="P523" s="27"/>
+      <x:c r="Q523" s="27"/>
+      <x:c r="R523" s="28"/>
+    </x:row>
+    <x:row r="524">
+      <x:c r="A524" s="29"/>
+      <x:c r="B524" s="30"/>
+      <x:c r="C524" s="30"/>
+      <x:c r="D524" s="30"/>
+      <x:c r="E524" s="30"/>
+      <x:c r="F524" s="30"/>
+      <x:c r="G524" s="30"/>
+      <x:c r="H524" s="30"/>
+      <x:c r="I524" s="30"/>
+      <x:c r="J524" s="30"/>
+      <x:c r="K524" s="30"/>
+      <x:c r="L524" s="30"/>
+      <x:c r="M524" s="30"/>
+      <x:c r="N524" s="30"/>
+      <x:c r="O524" s="30"/>
+      <x:c r="P524" s="30"/>
+      <x:c r="Q524" s="30"/>
+      <x:c r="R524" s="31"/>
+    </x:row>
+    <x:row r="525">
+      <x:c r="A525" s="44"/>
+      <x:c r="B525" s="45"/>
+      <x:c r="C525" s="45"/>
+      <x:c r="D525" s="45"/>
+      <x:c r="E525" s="45"/>
+      <x:c r="F525" s="45"/>
+      <x:c r="G525" s="45"/>
+      <x:c r="H525" s="45"/>
+      <x:c r="I525" s="45"/>
+      <x:c r="J525" s="45"/>
+      <x:c r="K525" s="45"/>
+      <x:c r="L525" s="45"/>
+      <x:c r="M525" s="45"/>
+      <x:c r="N525" s="45"/>
+      <x:c r="O525" s="45"/>
+      <x:c r="P525" s="45"/>
+      <x:c r="Q525" s="45"/>
+      <x:c r="R525" s="46"/>
+    </x:row>
+    <x:row r="526">
+      <x:c r="A526" s="47"/>
+      <x:c r="B526" s="48"/>
+      <x:c r="C526" s="48"/>
+      <x:c r="D526" s="48"/>
+      <x:c r="E526" s="48"/>
+      <x:c r="F526" s="48"/>
+      <x:c r="G526" s="48"/>
+      <x:c r="H526" s="48"/>
+      <x:c r="I526" s="48"/>
+      <x:c r="J526" s="48"/>
+      <x:c r="K526" s="48"/>
+      <x:c r="L526" s="48"/>
+      <x:c r="M526" s="48"/>
+      <x:c r="N526" s="48"/>
+      <x:c r="O526" s="48"/>
+      <x:c r="P526" s="48"/>
+      <x:c r="Q526" s="48"/>
+      <x:c r="R526" s="49"/>
+    </x:row>
+    <x:row r="527">
+      <x:c r="A527" s="47"/>
+      <x:c r="B527" s="48"/>
+      <x:c r="C527" s="48"/>
+      <x:c r="D527" s="48"/>
+      <x:c r="E527" s="48"/>
+      <x:c r="F527" s="48"/>
+      <x:c r="G527" s="48"/>
+      <x:c r="H527" s="48"/>
+      <x:c r="I527" s="48"/>
+      <x:c r="J527" s="48"/>
+      <x:c r="K527" s="48"/>
+      <x:c r="L527" s="48"/>
+      <x:c r="M527" s="48"/>
+      <x:c r="N527" s="48"/>
+      <x:c r="O527" s="48"/>
+      <x:c r="P527" s="48"/>
+      <x:c r="Q527" s="48"/>
+      <x:c r="R527" s="49"/>
+    </x:row>
+    <x:row r="528">
+      <x:c r="A528" s="47"/>
+      <x:c r="B528" s="48"/>
+      <x:c r="C528" s="48"/>
+      <x:c r="D528" s="48"/>
+      <x:c r="E528" s="48"/>
+      <x:c r="F528" s="48"/>
+      <x:c r="G528" s="48"/>
+      <x:c r="H528" s="48"/>
+      <x:c r="I528" s="48"/>
+      <x:c r="J528" s="48"/>
+      <x:c r="K528" s="48"/>
+      <x:c r="L528" s="48"/>
+      <x:c r="M528" s="48"/>
+      <x:c r="N528" s="48"/>
+      <x:c r="O528" s="48"/>
+      <x:c r="P528" s="48"/>
+      <x:c r="Q528" s="48"/>
+      <x:c r="R528" s="49"/>
+    </x:row>
+    <x:row r="529">
+      <x:c r="A529" s="47"/>
+      <x:c r="B529" s="48"/>
+      <x:c r="C529" s="48"/>
+      <x:c r="D529" s="48"/>
+      <x:c r="E529" s="48"/>
+      <x:c r="F529" s="48"/>
+      <x:c r="G529" s="48"/>
+      <x:c r="H529" s="48"/>
+      <x:c r="I529" s="48"/>
+      <x:c r="J529" s="48"/>
+      <x:c r="K529" s="48"/>
+      <x:c r="L529" s="48"/>
+      <x:c r="M529" s="48"/>
+      <x:c r="N529" s="48"/>
+      <x:c r="O529" s="48"/>
+      <x:c r="P529" s="48"/>
+      <x:c r="Q529" s="48"/>
+      <x:c r="R529" s="49"/>
+    </x:row>
+    <x:row r="530">
+      <x:c r="A530" s="47"/>
+      <x:c r="B530" s="48"/>
+      <x:c r="C530" s="48"/>
+      <x:c r="D530" s="48"/>
+      <x:c r="E530" s="48"/>
+      <x:c r="F530" s="48"/>
+      <x:c r="G530" s="48"/>
+      <x:c r="H530" s="48"/>
+      <x:c r="I530" s="48"/>
+      <x:c r="J530" s="48"/>
+      <x:c r="K530" s="48"/>
+      <x:c r="L530" s="48"/>
+      <x:c r="M530" s="48"/>
+      <x:c r="N530" s="48"/>
+      <x:c r="O530" s="48"/>
+      <x:c r="P530" s="48"/>
+      <x:c r="Q530" s="48"/>
+      <x:c r="R530" s="49"/>
+    </x:row>
+    <x:row r="531">
+      <x:c r="A531" s="47"/>
+      <x:c r="B531" s="48"/>
+      <x:c r="C531" s="48"/>
+      <x:c r="D531" s="48"/>
+      <x:c r="E531" s="48"/>
+      <x:c r="F531" s="48"/>
+      <x:c r="G531" s="48"/>
+      <x:c r="H531" s="48"/>
+      <x:c r="I531" s="48"/>
+      <x:c r="J531" s="48"/>
+      <x:c r="K531" s="48"/>
+      <x:c r="L531" s="48"/>
+      <x:c r="M531" s="48"/>
+      <x:c r="N531" s="48"/>
+      <x:c r="O531" s="48"/>
+      <x:c r="P531" s="48"/>
+      <x:c r="Q531" s="48"/>
+      <x:c r="R531" s="49"/>
+    </x:row>
+    <x:row r="532">
+      <x:c r="A532" s="47"/>
+      <x:c r="B532" s="48"/>
+      <x:c r="C532" s="48"/>
+      <x:c r="D532" s="48"/>
+      <x:c r="E532" s="48"/>
+      <x:c r="F532" s="48"/>
+      <x:c r="G532" s="48"/>
+      <x:c r="H532" s="48"/>
+      <x:c r="I532" s="48"/>
+      <x:c r="J532" s="48"/>
+      <x:c r="K532" s="48"/>
+      <x:c r="L532" s="48"/>
+      <x:c r="M532" s="48"/>
+      <x:c r="N532" s="48"/>
+      <x:c r="O532" s="48"/>
+      <x:c r="P532" s="48"/>
+      <x:c r="Q532" s="48"/>
+      <x:c r="R532" s="49"/>
+    </x:row>
+    <x:row r="533">
+      <x:c r="A533" s="47"/>
+      <x:c r="B533" s="48"/>
+      <x:c r="C533" s="48"/>
+      <x:c r="D533" s="48"/>
+      <x:c r="E533" s="48"/>
+      <x:c r="F533" s="48"/>
+      <x:c r="G533" s="48"/>
+      <x:c r="H533" s="48"/>
+      <x:c r="I533" s="48"/>
+      <x:c r="J533" s="48"/>
+      <x:c r="K533" s="48"/>
+      <x:c r="L533" s="48"/>
+      <x:c r="M533" s="48"/>
+      <x:c r="N533" s="48"/>
+      <x:c r="O533" s="48"/>
+      <x:c r="P533" s="48"/>
+      <x:c r="Q533" s="48"/>
+      <x:c r="R533" s="49"/>
+    </x:row>
+    <x:row r="534">
+      <x:c r="A534" s="47"/>
+      <x:c r="B534" s="48"/>
+      <x:c r="C534" s="48"/>
+      <x:c r="D534" s="48"/>
+      <x:c r="E534" s="48"/>
+      <x:c r="F534" s="48"/>
+      <x:c r="G534" s="48"/>
+      <x:c r="H534" s="48"/>
+      <x:c r="I534" s="48"/>
+      <x:c r="J534" s="48"/>
+      <x:c r="K534" s="48"/>
+      <x:c r="L534" s="48"/>
+      <x:c r="M534" s="48"/>
+      <x:c r="N534" s="48"/>
+      <x:c r="O534" s="48"/>
+      <x:c r="P534" s="48"/>
+      <x:c r="Q534" s="48"/>
+      <x:c r="R534" s="49"/>
+    </x:row>
+    <x:row r="535">
+      <x:c r="A535" s="47"/>
+      <x:c r="B535" s="48"/>
+      <x:c r="C535" s="48"/>
+      <x:c r="D535" s="48"/>
+      <x:c r="E535" s="48"/>
+      <x:c r="F535" s="48"/>
+      <x:c r="G535" s="48"/>
+      <x:c r="H535" s="48"/>
+      <x:c r="I535" s="48"/>
+      <x:c r="J535" s="48"/>
+      <x:c r="K535" s="48"/>
+      <x:c r="L535" s="48"/>
+      <x:c r="M535" s="48"/>
+      <x:c r="N535" s="48"/>
+      <x:c r="O535" s="48"/>
+      <x:c r="P535" s="48"/>
+      <x:c r="Q535" s="48"/>
+      <x:c r="R535" s="49"/>
+    </x:row>
+    <x:row r="536">
+      <x:c r="A536" s="47"/>
+      <x:c r="B536" s="48"/>
+      <x:c r="C536" s="48"/>
+      <x:c r="D536" s="48"/>
+      <x:c r="E536" s="48"/>
+      <x:c r="F536" s="48"/>
+      <x:c r="G536" s="48"/>
+      <x:c r="H536" s="48"/>
+      <x:c r="I536" s="48"/>
+      <x:c r="J536" s="48"/>
+      <x:c r="K536" s="48"/>
+      <x:c r="L536" s="48"/>
+      <x:c r="M536" s="48"/>
+      <x:c r="N536" s="48"/>
+      <x:c r="O536" s="48"/>
+      <x:c r="P536" s="48"/>
+      <x:c r="Q536" s="48"/>
+      <x:c r="R536" s="49"/>
+    </x:row>
+    <x:row r="537">
+      <x:c r="A537" s="47"/>
+      <x:c r="B537" s="48"/>
+      <x:c r="C537" s="48"/>
+      <x:c r="D537" s="48"/>
+      <x:c r="E537" s="48"/>
+      <x:c r="F537" s="48"/>
+      <x:c r="G537" s="48"/>
+      <x:c r="H537" s="48"/>
+      <x:c r="I537" s="48"/>
+      <x:c r="J537" s="48"/>
+      <x:c r="K537" s="48"/>
+      <x:c r="L537" s="48"/>
+      <x:c r="M537" s="48"/>
+      <x:c r="N537" s="48"/>
+      <x:c r="O537" s="48"/>
+      <x:c r="P537" s="48"/>
+      <x:c r="Q537" s="48"/>
+      <x:c r="R537" s="49"/>
+    </x:row>
+    <x:row r="538">
+      <x:c r="A538" s="47"/>
+      <x:c r="B538" s="48"/>
+      <x:c r="C538" s="48"/>
+      <x:c r="D538" s="48"/>
+      <x:c r="E538" s="48"/>
+      <x:c r="F538" s="48"/>
+      <x:c r="G538" s="48"/>
+      <x:c r="H538" s="48"/>
+      <x:c r="I538" s="48"/>
+      <x:c r="J538" s="48"/>
+      <x:c r="K538" s="48"/>
+      <x:c r="L538" s="48"/>
+      <x:c r="M538" s="48"/>
+      <x:c r="N538" s="48"/>
+      <x:c r="O538" s="48"/>
+      <x:c r="P538" s="48"/>
+      <x:c r="Q538" s="48"/>
+      <x:c r="R538" s="49"/>
+    </x:row>
+    <x:row r="539">
+      <x:c r="A539" s="47"/>
+      <x:c r="B539" s="48"/>
+      <x:c r="C539" s="48"/>
+      <x:c r="D539" s="48"/>
+      <x:c r="E539" s="48"/>
+      <x:c r="F539" s="48"/>
+      <x:c r="G539" s="48"/>
+      <x:c r="H539" s="48"/>
+      <x:c r="I539" s="48"/>
+      <x:c r="J539" s="48"/>
+      <x:c r="K539" s="48"/>
+      <x:c r="L539" s="48"/>
+      <x:c r="M539" s="48"/>
+      <x:c r="N539" s="48"/>
+      <x:c r="O539" s="48"/>
+      <x:c r="P539" s="48"/>
+      <x:c r="Q539" s="48"/>
+      <x:c r="R539" s="49"/>
+    </x:row>
+    <x:row r="540">
+      <x:c r="A540" s="47"/>
+      <x:c r="B540" s="48"/>
+      <x:c r="C540" s="48"/>
+      <x:c r="D540" s="48"/>
+      <x:c r="E540" s="48"/>
+      <x:c r="F540" s="48"/>
+      <x:c r="G540" s="48"/>
+      <x:c r="H540" s="48"/>
+      <x:c r="I540" s="48"/>
+      <x:c r="J540" s="48"/>
+      <x:c r="K540" s="48"/>
+      <x:c r="L540" s="48"/>
+      <x:c r="M540" s="48"/>
+      <x:c r="N540" s="48"/>
+      <x:c r="O540" s="48"/>
+      <x:c r="P540" s="48"/>
+      <x:c r="Q540" s="48"/>
+      <x:c r="R540" s="49"/>
+    </x:row>
+    <x:row r="541">
+      <x:c r="A541" s="47"/>
+      <x:c r="B541" s="48"/>
+      <x:c r="C541" s="48"/>
+      <x:c r="D541" s="48"/>
+      <x:c r="E541" s="48"/>
+      <x:c r="F541" s="48"/>
+      <x:c r="G541" s="48"/>
+      <x:c r="H541" s="48"/>
+      <x:c r="I541" s="48"/>
+      <x:c r="J541" s="48"/>
+      <x:c r="K541" s="48"/>
+      <x:c r="L541" s="48"/>
+      <x:c r="M541" s="48"/>
+      <x:c r="N541" s="48"/>
+      <x:c r="O541" s="48"/>
+      <x:c r="P541" s="48"/>
+      <x:c r="Q541" s="48"/>
+      <x:c r="R541" s="49"/>
+    </x:row>
+    <x:row r="542">
+      <x:c r="A542" s="47"/>
+      <x:c r="B542" s="48"/>
+      <x:c r="C542" s="48"/>
+      <x:c r="D542" s="48"/>
+      <x:c r="E542" s="48"/>
+      <x:c r="F542" s="48"/>
+      <x:c r="G542" s="48"/>
+      <x:c r="H542" s="48"/>
+      <x:c r="I542" s="48"/>
+      <x:c r="J542" s="48"/>
+      <x:c r="K542" s="48"/>
+      <x:c r="L542" s="48"/>
+      <x:c r="M542" s="48"/>
+      <x:c r="N542" s="48"/>
+      <x:c r="O542" s="48"/>
+      <x:c r="P542" s="48"/>
+      <x:c r="Q542" s="48"/>
+      <x:c r="R542" s="49"/>
+    </x:row>
+    <x:row r="543">
+      <x:c r="A543" s="47"/>
+      <x:c r="B543" s="48"/>
+      <x:c r="C543" s="48"/>
+      <x:c r="D543" s="48"/>
+      <x:c r="E543" s="48"/>
+      <x:c r="F543" s="48"/>
+      <x:c r="G543" s="48"/>
+      <x:c r="H543" s="48"/>
+      <x:c r="I543" s="48"/>
+      <x:c r="J543" s="48"/>
+      <x:c r="K543" s="48"/>
+      <x:c r="L543" s="48"/>
+      <x:c r="M543" s="48"/>
+      <x:c r="N543" s="48"/>
+      <x:c r="O543" s="48"/>
+      <x:c r="P543" s="48"/>
+      <x:c r="Q543" s="48"/>
+      <x:c r="R543" s="49"/>
+    </x:row>
+    <x:row r="544">
+      <x:c r="A544" s="50"/>
+      <x:c r="B544" s="51"/>
+      <x:c r="C544" s="51"/>
+      <x:c r="D544" s="51"/>
+      <x:c r="E544" s="51"/>
+      <x:c r="F544" s="51"/>
+      <x:c r="G544" s="51"/>
+      <x:c r="H544" s="51"/>
+      <x:c r="I544" s="51"/>
+      <x:c r="J544" s="51"/>
+      <x:c r="K544" s="51"/>
+      <x:c r="L544" s="51"/>
+      <x:c r="M544" s="51"/>
+      <x:c r="N544" s="51"/>
+      <x:c r="O544" s="51"/>
+      <x:c r="P544" s="51"/>
+      <x:c r="Q544" s="51"/>
+      <x:c r="R544" s="52"/>
+    </x:row>
+    <x:row r="545">
+      <x:c r="A545" s="61"/>
+      <x:c r="B545" s="62"/>
+      <x:c r="C545" s="62"/>
+      <x:c r="D545" s="62"/>
+      <x:c r="E545" s="62"/>
+      <x:c r="F545" s="62"/>
+      <x:c r="G545" s="62"/>
+      <x:c r="H545" s="62"/>
+      <x:c r="I545" s="62"/>
+      <x:c r="J545" s="62"/>
+      <x:c r="K545" s="62"/>
+      <x:c r="L545" s="62"/>
+      <x:c r="M545" s="62"/>
+      <x:c r="N545" s="62"/>
+      <x:c r="O545" s="62"/>
+      <x:c r="P545" s="62"/>
+      <x:c r="Q545" s="62"/>
+      <x:c r="R545" s="63"/>
+    </x:row>
+    <x:row r="546">
+      <x:c r="A546" s="64"/>
+      <x:c r="B546" s="65"/>
+      <x:c r="C546" s="65"/>
+      <x:c r="D546" s="65"/>
+      <x:c r="E546" s="65"/>
+      <x:c r="F546" s="65"/>
+      <x:c r="G546" s="65"/>
+      <x:c r="H546" s="65"/>
+      <x:c r="I546" s="65"/>
+      <x:c r="J546" s="65"/>
+      <x:c r="K546" s="65"/>
+      <x:c r="L546" s="65"/>
+      <x:c r="M546" s="65"/>
+      <x:c r="N546" s="65"/>
+      <x:c r="O546" s="65"/>
+      <x:c r="P546" s="65"/>
+      <x:c r="Q546" s="65"/>
+      <x:c r="R546" s="66"/>
+    </x:row>
+    <x:row r="547">
+      <x:c r="A547" s="64"/>
+      <x:c r="B547" s="65"/>
+      <x:c r="C547" s="65"/>
+      <x:c r="D547" s="65"/>
+      <x:c r="E547" s="65"/>
+      <x:c r="F547" s="65"/>
+      <x:c r="G547" s="65"/>
+      <x:c r="H547" s="65"/>
+      <x:c r="I547" s="65"/>
+      <x:c r="J547" s="65"/>
+      <x:c r="K547" s="65"/>
+      <x:c r="L547" s="65"/>
+      <x:c r="M547" s="65"/>
+      <x:c r="N547" s="65"/>
+      <x:c r="O547" s="65"/>
+      <x:c r="P547" s="65"/>
+      <x:c r="Q547" s="65"/>
+      <x:c r="R547" s="66"/>
+    </x:row>
+    <x:row r="548">
+      <x:c r="A548" s="64"/>
+      <x:c r="B548" s="65"/>
+      <x:c r="C548" s="65"/>
+      <x:c r="D548" s="65"/>
+      <x:c r="E548" s="65"/>
+      <x:c r="F548" s="65"/>
+      <x:c r="G548" s="65"/>
+      <x:c r="H548" s="65"/>
+      <x:c r="I548" s="65"/>
+      <x:c r="J548" s="65"/>
+      <x:c r="K548" s="65"/>
+      <x:c r="L548" s="65"/>
+      <x:c r="M548" s="65"/>
+      <x:c r="N548" s="65"/>
+      <x:c r="O548" s="65"/>
+      <x:c r="P548" s="65"/>
+      <x:c r="Q548" s="65"/>
+      <x:c r="R548" s="66"/>
+    </x:row>
+    <x:row r="549">
+      <x:c r="A549" s="64"/>
+      <x:c r="B549" s="65"/>
+      <x:c r="C549" s="65"/>
+      <x:c r="D549" s="65"/>
+      <x:c r="E549" s="65"/>
+      <x:c r="F549" s="65"/>
+      <x:c r="G549" s="65"/>
+      <x:c r="H549" s="65"/>
+      <x:c r="I549" s="65"/>
+      <x:c r="J549" s="65"/>
+      <x:c r="K549" s="65"/>
+      <x:c r="L549" s="65"/>
+      <x:c r="M549" s="65"/>
+      <x:c r="N549" s="65"/>
+      <x:c r="O549" s="65"/>
+      <x:c r="P549" s="65"/>
+      <x:c r="Q549" s="65"/>
+      <x:c r="R549" s="66"/>
+    </x:row>
+    <x:row r="550">
+      <x:c r="A550" s="64"/>
+      <x:c r="B550" s="65"/>
+      <x:c r="C550" s="65"/>
+      <x:c r="D550" s="65"/>
+      <x:c r="E550" s="65"/>
+      <x:c r="F550" s="65"/>
+      <x:c r="G550" s="65"/>
+      <x:c r="H550" s="65"/>
+      <x:c r="I550" s="65"/>
+      <x:c r="J550" s="65"/>
+      <x:c r="K550" s="65"/>
+      <x:c r="L550" s="65"/>
+      <x:c r="M550" s="65"/>
+      <x:c r="N550" s="65"/>
+      <x:c r="O550" s="65"/>
+      <x:c r="P550" s="65"/>
+      <x:c r="Q550" s="65"/>
+      <x:c r="R550" s="66"/>
+    </x:row>
+    <x:row r="551">
+      <x:c r="A551" s="64"/>
+      <x:c r="B551" s="65"/>
+      <x:c r="C551" s="65"/>
+      <x:c r="D551" s="65"/>
+      <x:c r="E551" s="65"/>
+      <x:c r="F551" s="65"/>
+      <x:c r="G551" s="65"/>
+      <x:c r="H551" s="65"/>
+      <x:c r="I551" s="65"/>
+      <x:c r="J551" s="65"/>
+      <x:c r="K551" s="65"/>
+      <x:c r="L551" s="65"/>
+      <x:c r="M551" s="65"/>
+      <x:c r="N551" s="65"/>
+      <x:c r="O551" s="65"/>
+      <x:c r="P551" s="65"/>
+      <x:c r="Q551" s="65"/>
+      <x:c r="R551" s="66"/>
+    </x:row>
+    <x:row r="552">
+      <x:c r="A552" s="64"/>
+      <x:c r="B552" s="65"/>
+      <x:c r="C552" s="65"/>
+      <x:c r="D552" s="65"/>
+      <x:c r="E552" s="65"/>
+      <x:c r="F552" s="65"/>
+      <x:c r="G552" s="65"/>
+      <x:c r="H552" s="65"/>
+      <x:c r="I552" s="65"/>
+      <x:c r="J552" s="65"/>
+      <x:c r="K552" s="65"/>
+      <x:c r="L552" s="65"/>
+      <x:c r="M552" s="65"/>
+      <x:c r="N552" s="65"/>
+      <x:c r="O552" s="65"/>
+      <x:c r="P552" s="65"/>
+      <x:c r="Q552" s="65"/>
+      <x:c r="R552" s="66"/>
+    </x:row>
+    <x:row r="553">
+      <x:c r="A553" s="64"/>
+      <x:c r="B553" s="65"/>
+      <x:c r="C553" s="65"/>
+      <x:c r="D553" s="65"/>
+      <x:c r="E553" s="65"/>
+      <x:c r="F553" s="65"/>
+      <x:c r="G553" s="65"/>
+      <x:c r="H553" s="65"/>
+      <x:c r="I553" s="65"/>
+      <x:c r="J553" s="65"/>
+      <x:c r="K553" s="65"/>
+      <x:c r="L553" s="65"/>
+      <x:c r="M553" s="65"/>
+      <x:c r="N553" s="65"/>
+      <x:c r="O553" s="65"/>
+      <x:c r="P553" s="65"/>
+      <x:c r="Q553" s="65"/>
+      <x:c r="R553" s="66"/>
+    </x:row>
+    <x:row r="554">
+      <x:c r="A554" s="64"/>
+      <x:c r="B554" s="65"/>
+      <x:c r="C554" s="65"/>
+      <x:c r="D554" s="65"/>
+      <x:c r="E554" s="65"/>
+      <x:c r="F554" s="65"/>
+      <x:c r="G554" s="65"/>
+      <x:c r="H554" s="65"/>
+      <x:c r="I554" s="65"/>
+      <x:c r="J554" s="65"/>
+      <x:c r="K554" s="65"/>
+      <x:c r="L554" s="65"/>
+      <x:c r="M554" s="65"/>
+      <x:c r="N554" s="65"/>
+      <x:c r="O554" s="65"/>
+      <x:c r="P554" s="65"/>
+      <x:c r="Q554" s="65"/>
+      <x:c r="R554" s="66"/>
+    </x:row>
+    <x:row r="555">
+      <x:c r="A555" s="64"/>
+      <x:c r="B555" s="65"/>
+      <x:c r="C555" s="65"/>
+      <x:c r="D555" s="65"/>
+      <x:c r="E555" s="65"/>
+      <x:c r="F555" s="65"/>
+      <x:c r="G555" s="65"/>
+      <x:c r="H555" s="65"/>
+      <x:c r="I555" s="65"/>
+      <x:c r="J555" s="65"/>
+      <x:c r="K555" s="65"/>
+      <x:c r="L555" s="65"/>
+      <x:c r="M555" s="65"/>
+      <x:c r="N555" s="65"/>
+      <x:c r="O555" s="65"/>
+      <x:c r="P555" s="65"/>
+      <x:c r="Q555" s="65"/>
+      <x:c r="R555" s="66"/>
+    </x:row>
+    <x:row r="556">
+      <x:c r="A556" s="64"/>
+      <x:c r="B556" s="65"/>
+      <x:c r="C556" s="65"/>
+      <x:c r="D556" s="65"/>
+      <x:c r="E556" s="65"/>
+      <x:c r="F556" s="65"/>
+      <x:c r="G556" s="65"/>
+      <x:c r="H556" s="65"/>
+      <x:c r="I556" s="65"/>
+      <x:c r="J556" s="65"/>
+      <x:c r="K556" s="65"/>
+      <x:c r="L556" s="65"/>
+      <x:c r="M556" s="65"/>
+      <x:c r="N556" s="65"/>
+      <x:c r="O556" s="65"/>
+      <x:c r="P556" s="65"/>
+      <x:c r="Q556" s="65"/>
+      <x:c r="R556" s="66"/>
+    </x:row>
+    <x:row r="557">
+      <x:c r="A557" s="64"/>
+      <x:c r="B557" s="65"/>
+      <x:c r="C557" s="65"/>
+      <x:c r="D557" s="65"/>
+      <x:c r="E557" s="65"/>
+      <x:c r="F557" s="65"/>
+      <x:c r="G557" s="65"/>
+      <x:c r="H557" s="65"/>
+      <x:c r="I557" s="65"/>
+      <x:c r="J557" s="65"/>
+      <x:c r="K557" s="65"/>
+      <x:c r="L557" s="65"/>
+      <x:c r="M557" s="65"/>
+      <x:c r="N557" s="65"/>
+      <x:c r="O557" s="65"/>
+      <x:c r="P557" s="65"/>
+      <x:c r="Q557" s="65"/>
+      <x:c r="R557" s="66"/>
+    </x:row>
+    <x:row r="558">
+      <x:c r="A558" s="64"/>
+      <x:c r="B558" s="65"/>
+      <x:c r="C558" s="65"/>
+      <x:c r="D558" s="65"/>
+      <x:c r="E558" s="65"/>
+      <x:c r="F558" s="65"/>
+      <x:c r="G558" s="65"/>
+      <x:c r="H558" s="65"/>
+      <x:c r="I558" s="65"/>
+      <x:c r="J558" s="65"/>
+      <x:c r="K558" s="65"/>
+      <x:c r="L558" s="65"/>
+      <x:c r="M558" s="65"/>
+      <x:c r="N558" s="65"/>
+      <x:c r="O558" s="65"/>
+      <x:c r="P558" s="65"/>
+      <x:c r="Q558" s="65"/>
+      <x:c r="R558" s="66"/>
+    </x:row>
+    <x:row r="559">
+      <x:c r="A559" s="64"/>
+      <x:c r="B559" s="65"/>
+      <x:c r="C559" s="65"/>
+      <x:c r="D559" s="65"/>
+      <x:c r="E559" s="65"/>
+      <x:c r="F559" s="65"/>
+      <x:c r="G559" s="65"/>
+      <x:c r="H559" s="65"/>
+      <x:c r="I559" s="65"/>
+      <x:c r="J559" s="65"/>
+      <x:c r="K559" s="65"/>
+      <x:c r="L559" s="65"/>
+      <x:c r="M559" s="65"/>
+      <x:c r="N559" s="65"/>
+      <x:c r="O559" s="65"/>
+      <x:c r="P559" s="65"/>
+      <x:c r="Q559" s="65"/>
+      <x:c r="R559" s="66"/>
+    </x:row>
+    <x:row r="560">
+      <x:c r="A560" s="64"/>
+      <x:c r="B560" s="65"/>
+      <x:c r="C560" s="65"/>
+      <x:c r="D560" s="65"/>
+      <x:c r="E560" s="65"/>
+      <x:c r="F560" s="65"/>
+      <x:c r="G560" s="65"/>
+      <x:c r="H560" s="65"/>
+      <x:c r="I560" s="65"/>
+      <x:c r="J560" s="65"/>
+      <x:c r="K560" s="65"/>
+      <x:c r="L560" s="65"/>
+      <x:c r="M560" s="65"/>
+      <x:c r="N560" s="65"/>
+      <x:c r="O560" s="65"/>
+      <x:c r="P560" s="65"/>
+      <x:c r="Q560" s="65"/>
+      <x:c r="R560" s="66"/>
+    </x:row>
+    <x:row r="561">
+      <x:c r="A561" s="64"/>
+      <x:c r="B561" s="65"/>
+      <x:c r="C561" s="65"/>
+      <x:c r="D561" s="65"/>
+      <x:c r="E561" s="65"/>
+      <x:c r="F561" s="65"/>
+      <x:c r="G561" s="65"/>
+      <x:c r="H561" s="65"/>
+      <x:c r="I561" s="65"/>
+      <x:c r="J561" s="65"/>
+      <x:c r="K561" s="65"/>
+      <x:c r="L561" s="65"/>
+      <x:c r="M561" s="65"/>
+      <x:c r="N561" s="65"/>
+      <x:c r="O561" s="65"/>
+      <x:c r="P561" s="65"/>
+      <x:c r="Q561" s="65"/>
+      <x:c r="R561" s="66"/>
+    </x:row>
+    <x:row r="562">
+      <x:c r="A562" s="64"/>
+      <x:c r="B562" s="65"/>
+      <x:c r="C562" s="65"/>
+      <x:c r="D562" s="65"/>
+      <x:c r="E562" s="65"/>
+      <x:c r="F562" s="65"/>
+      <x:c r="G562" s="65"/>
+      <x:c r="H562" s="65"/>
+      <x:c r="I562" s="65"/>
+      <x:c r="J562" s="65"/>
+      <x:c r="K562" s="65"/>
+      <x:c r="L562" s="65"/>
+      <x:c r="M562" s="65"/>
+      <x:c r="N562" s="65"/>
+      <x:c r="O562" s="65"/>
+      <x:c r="P562" s="65"/>
+      <x:c r="Q562" s="65"/>
+      <x:c r="R562" s="66"/>
+    </x:row>
+    <x:row r="563">
+      <x:c r="A563" s="64"/>
+      <x:c r="B563" s="65"/>
+      <x:c r="C563" s="65"/>
+      <x:c r="D563" s="65"/>
+      <x:c r="E563" s="65"/>
+      <x:c r="F563" s="65"/>
+      <x:c r="G563" s="65"/>
+      <x:c r="H563" s="65"/>
+      <x:c r="I563" s="65"/>
+      <x:c r="J563" s="65"/>
+      <x:c r="K563" s="65"/>
+      <x:c r="L563" s="65"/>
+      <x:c r="M563" s="65"/>
+      <x:c r="N563" s="65"/>
+      <x:c r="O563" s="65"/>
+      <x:c r="P563" s="65"/>
+      <x:c r="Q563" s="65"/>
+      <x:c r="R563" s="66"/>
+    </x:row>
+    <x:row r="564">
+      <x:c r="A564" s="67"/>
+      <x:c r="B564" s="68"/>
+      <x:c r="C564" s="68"/>
+      <x:c r="D564" s="68"/>
+      <x:c r="E564" s="68"/>
+      <x:c r="F564" s="68"/>
+      <x:c r="G564" s="68"/>
+      <x:c r="H564" s="68"/>
+      <x:c r="I564" s="68"/>
+      <x:c r="J564" s="68"/>
+      <x:c r="K564" s="68"/>
+      <x:c r="L564" s="68"/>
+      <x:c r="M564" s="68"/>
+      <x:c r="N564" s="68"/>
+      <x:c r="O564" s="68"/>
+      <x:c r="P564" s="68"/>
+      <x:c r="Q564" s="68"/>
+      <x:c r="R564" s="69"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="6">
@@ -11438,10 +13271,18 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="12"/>
-      <x:c r="B11" s="12"/>
-      <x:c r="C11" s="12"/>
-      <x:c r="D11" s="12"/>
+      <x:c r="A11" s="70" t="str">
+        <x:v>ui.bg.archive</x:v>
+      </x:c>
+      <x:c r="B11" s="70" t="str">
+        <x:v>res://assets/helltaker/backgrounds/chapterBG0008.png</x:v>
+      </x:c>
+      <x:c r="C11" s="70" t="str">
+        <x:v>编队与图鉴背景</x:v>
+      </x:c>
+      <x:c r="D11" s="70" t="str">
+        <x:v>UI背景</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="12"/>
@@ -13051,242 +14892,612 @@
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="12"/>
-      <x:c r="B26" s="14"/>
-      <x:c r="C26" s="14"/>
-      <x:c r="D26" s="14"/>
-      <x:c r="E26" s="14"/>
-      <x:c r="F26" s="12"/>
-      <x:c r="G26" s="12"/>
-      <x:c r="H26" s="13"/>
-      <x:c r="I26" s="14"/>
-      <x:c r="J26" s="14"/>
-      <x:c r="K26" s="14"/>
-      <x:c r="L26" s="14"/>
-      <x:c r="M26" s="14"/>
-      <x:c r="N26" s="13"/>
-      <x:c r="O26" s="14"/>
+      <x:c r="A26" s="21" t="str">
+        <x:v>squad_button</x:v>
+      </x:c>
+      <x:c r="B26" s="20" t="n">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="C26" s="20" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D26" s="20" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="E26" s="20" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F26" s="19" t="str"/>
+      <x:c r="G26" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="str">
+        <x:v>编队  [F3]</x:v>
+      </x:c>
+      <x:c r="I26" s="20" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="J26" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K26" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N26" s="20" t="str">
+        <x:v>战斗顶部编队入口</x:v>
+      </x:c>
+      <x:c r="O26" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="12"/>
-      <x:c r="B27" s="14"/>
-      <x:c r="C27" s="14"/>
-      <x:c r="D27" s="14"/>
-      <x:c r="E27" s="14"/>
-      <x:c r="F27" s="12"/>
-      <x:c r="G27" s="12"/>
-      <x:c r="H27" s="13"/>
-      <x:c r="I27" s="14"/>
-      <x:c r="J27" s="14"/>
-      <x:c r="K27" s="14"/>
-      <x:c r="L27" s="14"/>
-      <x:c r="M27" s="14"/>
-      <x:c r="N27" s="13"/>
-      <x:c r="O27" s="14"/>
+      <x:c r="A27" s="21" t="str">
+        <x:v>squad_background</x:v>
+      </x:c>
+      <x:c r="B27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D27" s="20" t="n">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="E27" s="20" t="n">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>ui.bg.archive</x:v>
+      </x:c>
+      <x:c r="G27" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H27" s="19" t="str"/>
+      <x:c r="I27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M27" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N27" s="20" t="str">
+        <x:v>编队页背景</x:v>
+      </x:c>
+      <x:c r="O27" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="12"/>
-      <x:c r="B28" s="14"/>
-      <x:c r="C28" s="14"/>
-      <x:c r="D28" s="14"/>
-      <x:c r="E28" s="14"/>
-      <x:c r="F28" s="12"/>
-      <x:c r="G28" s="12"/>
-      <x:c r="H28" s="13"/>
-      <x:c r="I28" s="14"/>
-      <x:c r="J28" s="14"/>
-      <x:c r="K28" s="14"/>
-      <x:c r="L28" s="14"/>
-      <x:c r="M28" s="14"/>
-      <x:c r="N28" s="13"/>
-      <x:c r="O28" s="14"/>
+      <x:c r="A28" s="21" t="str">
+        <x:v>squad_frame</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C28" s="20" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D28" s="20" t="n">
+        <x:v>1136</x:v>
+      </x:c>
+      <x:c r="E28" s="20" t="n">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="F28" s="19" t="str"/>
+      <x:c r="G28" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H28" s="19" t="str"/>
+      <x:c r="I28" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N28" s="20" t="str">
+        <x:v>编队页主框</x:v>
+      </x:c>
+      <x:c r="O28" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="12"/>
-      <x:c r="B29" s="14"/>
-      <x:c r="C29" s="14"/>
-      <x:c r="D29" s="14"/>
-      <x:c r="E29" s="14"/>
-      <x:c r="F29" s="12"/>
-      <x:c r="G29" s="12"/>
-      <x:c r="H29" s="13"/>
-      <x:c r="I29" s="14"/>
-      <x:c r="J29" s="14"/>
-      <x:c r="K29" s="14"/>
-      <x:c r="L29" s="14"/>
-      <x:c r="M29" s="14"/>
-      <x:c r="N29" s="13"/>
-      <x:c r="O29" s="14"/>
+      <x:c r="A29" s="21" t="str">
+        <x:v>squad_title</x:v>
+      </x:c>
+      <x:c r="B29" s="20" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C29" s="20" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D29" s="20" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="E29" s="20" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F29" s="19" t="str"/>
+      <x:c r="G29" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H29" s="19" t="str"/>
+      <x:c r="I29" s="20" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J29" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M29" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N29" s="20" t="str">
+        <x:v>下一关标题</x:v>
+      </x:c>
+      <x:c r="O29" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="12"/>
-      <x:c r="B30" s="14"/>
-      <x:c r="C30" s="14"/>
-      <x:c r="D30" s="14"/>
-      <x:c r="E30" s="14"/>
-      <x:c r="F30" s="12"/>
-      <x:c r="G30" s="12"/>
-      <x:c r="H30" s="13"/>
-      <x:c r="I30" s="14"/>
-      <x:c r="J30" s="14"/>
-      <x:c r="K30" s="14"/>
-      <x:c r="L30" s="14"/>
-      <x:c r="M30" s="14"/>
-      <x:c r="N30" s="13"/>
-      <x:c r="O30" s="14"/>
+      <x:c r="A30" s="21" t="str">
+        <x:v>squad_subtitle</x:v>
+      </x:c>
+      <x:c r="B30" s="20" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C30" s="20" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="D30" s="20" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="E30" s="20" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F30" s="19" t="str"/>
+      <x:c r="G30" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="str"/>
+      <x:c r="I30" s="20" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="J30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N30" s="20" t="str">
+        <x:v>解锁提示</x:v>
+      </x:c>
+      <x:c r="O30" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
-      <x:c r="A31" s="12"/>
-      <x:c r="B31" s="14"/>
-      <x:c r="C31" s="14"/>
-      <x:c r="D31" s="14"/>
-      <x:c r="E31" s="14"/>
-      <x:c r="F31" s="12"/>
-      <x:c r="G31" s="12"/>
-      <x:c r="H31" s="13"/>
-      <x:c r="I31" s="14"/>
-      <x:c r="J31" s="14"/>
-      <x:c r="K31" s="14"/>
-      <x:c r="L31" s="14"/>
-      <x:c r="M31" s="14"/>
-      <x:c r="N31" s="13"/>
-      <x:c r="O31" s="14"/>
+      <x:c r="A31" s="21" t="str">
+        <x:v>squad_confirm</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="n">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="n">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="F31" s="19" t="str"/>
+      <x:c r="G31" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H31" s="19" t="str">
+        <x:v>确认编队并进入下一关   →</x:v>
+      </x:c>
+      <x:c r="I31" s="20" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J31" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K31" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M31" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N31" s="20" t="str">
+        <x:v>确认按钮</x:v>
+      </x:c>
+      <x:c r="O31" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
-      <x:c r="A32" s="12"/>
-      <x:c r="B32" s="14"/>
-      <x:c r="C32" s="14"/>
-      <x:c r="D32" s="14"/>
-      <x:c r="E32" s="14"/>
-      <x:c r="F32" s="12"/>
-      <x:c r="G32" s="12"/>
-      <x:c r="H32" s="13"/>
-      <x:c r="I32" s="14"/>
-      <x:c r="J32" s="14"/>
-      <x:c r="K32" s="14"/>
-      <x:c r="L32" s="14"/>
-      <x:c r="M32" s="14"/>
-      <x:c r="N32" s="13"/>
-      <x:c r="O32" s="14"/>
+      <x:c r="A32" s="21" t="str">
+        <x:v>squad_character_1</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F32" s="19" t="str"/>
+      <x:c r="G32" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H32" s="19" t="str"/>
+      <x:c r="I32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N32" s="20" t="str">
+        <x:v>角色槽位 1</x:v>
+      </x:c>
+      <x:c r="O32" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
-      <x:c r="A33" s="12"/>
-      <x:c r="B33" s="14"/>
-      <x:c r="C33" s="14"/>
-      <x:c r="D33" s="14"/>
-      <x:c r="E33" s="14"/>
-      <x:c r="F33" s="12"/>
-      <x:c r="G33" s="12"/>
-      <x:c r="H33" s="13"/>
-      <x:c r="I33" s="14"/>
-      <x:c r="J33" s="14"/>
-      <x:c r="K33" s="14"/>
-      <x:c r="L33" s="14"/>
-      <x:c r="M33" s="14"/>
-      <x:c r="N33" s="13"/>
-      <x:c r="O33" s="14"/>
+      <x:c r="A33" s="21" t="str">
+        <x:v>squad_character_2</x:v>
+      </x:c>
+      <x:c r="B33" s="20" t="n">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="C33" s="20" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D33" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E33" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F33" s="19" t="str"/>
+      <x:c r="G33" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H33" s="19" t="str"/>
+      <x:c r="I33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N33" s="20" t="str">
+        <x:v>角色槽位 2</x:v>
+      </x:c>
+      <x:c r="O33" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
-      <x:c r="A34" s="12"/>
-      <x:c r="B34" s="14"/>
-      <x:c r="C34" s="14"/>
-      <x:c r="D34" s="14"/>
-      <x:c r="E34" s="14"/>
-      <x:c r="F34" s="12"/>
-      <x:c r="G34" s="12"/>
-      <x:c r="H34" s="13"/>
-      <x:c r="I34" s="14"/>
-      <x:c r="J34" s="14"/>
-      <x:c r="K34" s="14"/>
-      <x:c r="L34" s="14"/>
-      <x:c r="M34" s="14"/>
-      <x:c r="N34" s="13"/>
-      <x:c r="O34" s="14"/>
+      <x:c r="A34" s="21" t="str">
+        <x:v>squad_character_3</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="n">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C34" s="20" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F34" s="19" t="str"/>
+      <x:c r="G34" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H34" s="19" t="str"/>
+      <x:c r="I34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="20" t="str">
+        <x:v>角色槽位 3</x:v>
+      </x:c>
+      <x:c r="O34" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="30" customHeight="1">
-      <x:c r="A35" s="12"/>
-      <x:c r="B35" s="14"/>
-      <x:c r="C35" s="14"/>
-      <x:c r="D35" s="14"/>
-      <x:c r="E35" s="14"/>
-      <x:c r="F35" s="12"/>
-      <x:c r="G35" s="12"/>
-      <x:c r="H35" s="13"/>
-      <x:c r="I35" s="14"/>
-      <x:c r="J35" s="14"/>
-      <x:c r="K35" s="14"/>
-      <x:c r="L35" s="14"/>
-      <x:c r="M35" s="14"/>
-      <x:c r="N35" s="13"/>
-      <x:c r="O35" s="14"/>
+      <x:c r="A35" s="21" t="str">
+        <x:v>squad_character_4</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="n">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="C35" s="20" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D35" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E35" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F35" s="19" t="str"/>
+      <x:c r="G35" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H35" s="19" t="str"/>
+      <x:c r="I35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="20" t="str">
+        <x:v>角色槽位 4</x:v>
+      </x:c>
+      <x:c r="O35" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="30" customHeight="1">
-      <x:c r="A36" s="12"/>
-      <x:c r="B36" s="14"/>
-      <x:c r="C36" s="14"/>
-      <x:c r="D36" s="14"/>
-      <x:c r="E36" s="14"/>
-      <x:c r="F36" s="12"/>
-      <x:c r="G36" s="12"/>
-      <x:c r="H36" s="13"/>
-      <x:c r="I36" s="14"/>
-      <x:c r="J36" s="14"/>
-      <x:c r="K36" s="14"/>
-      <x:c r="L36" s="14"/>
-      <x:c r="M36" s="14"/>
-      <x:c r="N36" s="13"/>
-      <x:c r="O36" s="14"/>
+      <x:c r="A36" s="21" t="str">
+        <x:v>squad_character_5</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C36" s="20" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D36" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E36" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F36" s="19" t="str"/>
+      <x:c r="G36" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H36" s="19" t="str"/>
+      <x:c r="I36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="20" t="str">
+        <x:v>角色槽位 5</x:v>
+      </x:c>
+      <x:c r="O36" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="12"/>
-      <x:c r="B37" s="14"/>
-      <x:c r="C37" s="14"/>
-      <x:c r="D37" s="14"/>
-      <x:c r="E37" s="14"/>
-      <x:c r="F37" s="12"/>
-      <x:c r="G37" s="12"/>
-      <x:c r="H37" s="13"/>
-      <x:c r="I37" s="14"/>
-      <x:c r="J37" s="14"/>
-      <x:c r="K37" s="14"/>
-      <x:c r="L37" s="14"/>
-      <x:c r="M37" s="14"/>
-      <x:c r="N37" s="13"/>
-      <x:c r="O37" s="14"/>
+      <x:c r="A37" s="21" t="str">
+        <x:v>squad_character_6</x:v>
+      </x:c>
+      <x:c r="B37" s="20" t="n">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="C37" s="20" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D37" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E37" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F37" s="19" t="str"/>
+      <x:c r="G37" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H37" s="19" t="str"/>
+      <x:c r="I37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="20" t="str">
+        <x:v>角色槽位 6</x:v>
+      </x:c>
+      <x:c r="O37" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="12"/>
-      <x:c r="B38" s="14"/>
-      <x:c r="C38" s="14"/>
-      <x:c r="D38" s="14"/>
-      <x:c r="E38" s="14"/>
-      <x:c r="F38" s="12"/>
-      <x:c r="G38" s="12"/>
-      <x:c r="H38" s="13"/>
-      <x:c r="I38" s="14"/>
-      <x:c r="J38" s="14"/>
-      <x:c r="K38" s="14"/>
-      <x:c r="L38" s="14"/>
-      <x:c r="M38" s="14"/>
-      <x:c r="N38" s="13"/>
-      <x:c r="O38" s="14"/>
+      <x:c r="A38" s="21" t="str">
+        <x:v>squad_character_7</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="n">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C38" s="20" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D38" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E38" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F38" s="19" t="str"/>
+      <x:c r="G38" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H38" s="19" t="str"/>
+      <x:c r="I38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="20" t="str">
+        <x:v>角色槽位 7</x:v>
+      </x:c>
+      <x:c r="O38" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="30" customHeight="1">
-      <x:c r="A39" s="12"/>
-      <x:c r="B39" s="14"/>
-      <x:c r="C39" s="14"/>
-      <x:c r="D39" s="14"/>
-      <x:c r="E39" s="14"/>
-      <x:c r="F39" s="12"/>
-      <x:c r="G39" s="12"/>
-      <x:c r="H39" s="13"/>
-      <x:c r="I39" s="14"/>
-      <x:c r="J39" s="14"/>
-      <x:c r="K39" s="14"/>
-      <x:c r="L39" s="14"/>
-      <x:c r="M39" s="14"/>
-      <x:c r="N39" s="13"/>
-      <x:c r="O39" s="14"/>
+      <x:c r="A39" s="21" t="str">
+        <x:v>squad_character_8</x:v>
+      </x:c>
+      <x:c r="B39" s="20" t="n">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="C39" s="20" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D39" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E39" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F39" s="19" t="str"/>
+      <x:c r="G39" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H39" s="19" t="str"/>
+      <x:c r="I39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="20" t="str">
+        <x:v>角色槽位 8</x:v>
+      </x:c>
+      <x:c r="O39" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="30" customHeight="1">
       <x:c r="A40" s="12"/>

</xml_diff>

<commit_message>
feat: add mission select and persistent records
</commit_message>
<xml_diff>
--- a/content/game_config.xlsx
+++ b/content/game_config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R5a6efd7a93fb4985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="R1ac26bf8e5574af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="R274f2f6833b64486"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="R63a0c9a1e0664d86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R15dbab3584914843"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="Rf4dbd024d322463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="R34c7f9dc8ff244f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="Rc3e9e8734fcb492e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -86,6 +86,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF8DE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -167,7 +172,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -315,6 +320,28 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -722,6 +749,14 @@
         <x:v>UI表的squad_开头控件可修改位置、尺寸、文字和素材；游戏中按F3打开编队。</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="55" t="str">
+        <x:v>关卡选择</x:v>
+      </x:c>
+      <x:c r="B27" s="56" t="str">
+        <x:v>UI表的stage_开头控件可修改关卡入口与选择页；游戏中按F4打开已解锁地图。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1824,674 +1859,674 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="57" t="n">
+      <x:c r="A22" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B22" s="58" t="str">
+      <x:c r="B22" s="73" t="str">
         <x:v>mode1_opening</x:v>
       </x:c>
-      <x:c r="C22" s="57" t="n">
+      <x:c r="C22" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D22" s="58" t="str">
+      <x:c r="D22" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E22" s="58" t="str">
+      <x:c r="E22" s="73" t="str">
         <x:v>裂隙已经越过警戒线。元素尚未回应我，但剑还在手里。</x:v>
       </x:c>
-      <x:c r="F22" s="58" t="str">
+      <x:c r="F22" s="73" t="str">
         <x:v>saria</x:v>
       </x:c>
-      <x:c r="G22" s="58" t="str">
+      <x:c r="G22" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H22" s="57" t="n">
+      <x:c r="H22" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I22" s="57" t="n">
+      <x:c r="I22" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J22" s="59" t="n">
+      <x:c r="J22" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K22" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L22" s="58" t="str">
+      <x:c r="K22" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M22" s="58" t="str">
+      <x:c r="M22" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N22" s="57" t="n">
+      <x:c r="N22" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O22" s="57" t="n">
+      <x:c r="O22" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P22" s="59" t="n">
+      <x:c r="P22" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q22" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R22" s="58" t="str">
+      <x:c r="Q22" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R22" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="57" t="n">
+      <x:c r="A23" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B23" s="58" t="str">
+      <x:c r="B23" s="73" t="str">
         <x:v>mode1_opening</x:v>
       </x:c>
-      <x:c r="C23" s="57" t="n">
+      <x:c r="C23" s="72" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D23" s="58" t="str">
+      <x:c r="D23" s="73" t="str">
         <x:v>通讯员</x:v>
       </x:c>
-      <x:c r="E23" s="58" t="str">
+      <x:c r="E23" s="73" t="str">
         <x:v>水晶会收集敌人的残响。每次升级都能改写攻击方式，弹道与支援也会随构筑增长。</x:v>
       </x:c>
-      <x:c r="F23" s="58" t="str">
+      <x:c r="F23" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="G23" s="58" t="str">
+      <x:c r="G23" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H23" s="57" t="n">
+      <x:c r="H23" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I23" s="57" t="n">
+      <x:c r="I23" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J23" s="59" t="n">
+      <x:c r="J23" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K23" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L23" s="58" t="str">
+      <x:c r="K23" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" s="73" t="str">
         <x:v>saria</x:v>
       </x:c>
-      <x:c r="M23" s="58" t="str">
+      <x:c r="M23" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N23" s="57" t="n">
+      <x:c r="N23" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O23" s="57" t="n">
+      <x:c r="O23" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P23" s="59" t="n">
+      <x:c r="P23" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q23" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R23" s="58" t="str">
+      <x:c r="Q23" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R23" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="57" t="n">
+      <x:c r="A24" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B24" s="58" t="str">
+      <x:c r="B24" s="73" t="str">
         <x:v>mode1_opening</x:v>
       </x:c>
-      <x:c r="C24" s="57" t="n">
+      <x:c r="C24" s="72" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D24" s="58" t="str">
+      <x:c r="D24" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E24" s="58" t="str">
+      <x:c r="E24" s="73" t="str">
         <x:v>那就从这里开始。守住五分半，把右侧涌来的东西全部送回去。</x:v>
       </x:c>
-      <x:c r="F24" s="58" t="str">
+      <x:c r="F24" s="73" t="str">
         <x:v>saria-soft</x:v>
       </x:c>
-      <x:c r="G24" s="58" t="str">
+      <x:c r="G24" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H24" s="57" t="n">
+      <x:c r="H24" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I24" s="57" t="n">
+      <x:c r="I24" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J24" s="59" t="n">
+      <x:c r="J24" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K24" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L24" s="58" t="str">
+      <x:c r="K24" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M24" s="58" t="str">
+      <x:c r="M24" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N24" s="57" t="n">
+      <x:c r="N24" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O24" s="57" t="n">
+      <x:c r="O24" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P24" s="59" t="n">
+      <x:c r="P24" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q24" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R24" s="58" t="str">
+      <x:c r="Q24" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R24" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="57" t="n">
+      <x:c r="A25" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B25" s="58" t="str">
+      <x:c r="B25" s="73" t="str">
         <x:v>mode1_won</x:v>
       </x:c>
-      <x:c r="C25" s="57" t="n">
+      <x:c r="C25" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D25" s="58" t="str">
+      <x:c r="D25" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E25" s="58" t="str">
+      <x:c r="E25" s="73" t="str">
         <x:v>第一道裂隙关闭了。水晶记录下了这次构筑，下一关会有新的同伴回应。</x:v>
       </x:c>
-      <x:c r="F25" s="58" t="str">
+      <x:c r="F25" s="73" t="str">
         <x:v>saria-soft</x:v>
       </x:c>
-      <x:c r="G25" s="58" t="str">
+      <x:c r="G25" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H25" s="57" t="n">
+      <x:c r="H25" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I25" s="57" t="n">
+      <x:c r="I25" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J25" s="59" t="n">
+      <x:c r="J25" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K25" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L25" s="58" t="str">
+      <x:c r="K25" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M25" s="58" t="str">
+      <x:c r="M25" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N25" s="57" t="n">
+      <x:c r="N25" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O25" s="57" t="n">
+      <x:c r="O25" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P25" s="59" t="n">
+      <x:c r="P25" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q25" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R25" s="58" t="str">
+      <x:c r="Q25" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R25" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="57" t="n">
+      <x:c r="A26" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B26" s="58" t="str">
+      <x:c r="B26" s="73" t="str">
         <x:v>mode1_stage2_opening</x:v>
       </x:c>
-      <x:c r="C26" s="57" t="n">
+      <x:c r="C26" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D26" s="58" t="str">
+      <x:c r="D26" s="73" t="str">
         <x:v>宵宫</x:v>
       </x:c>
-      <x:c r="E26" s="58" t="str">
+      <x:c r="E26" s="73" t="str">
         <x:v>通讯接通。第二道裂隙已经变成赤潮，我从高台提供火力。</x:v>
       </x:c>
-      <x:c r="F26" s="58" t="str">
+      <x:c r="F26" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="G26" s="58" t="str">
+      <x:c r="G26" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H26" s="57" t="n">
+      <x:c r="H26" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I26" s="57" t="n">
+      <x:c r="I26" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J26" s="59" t="n">
+      <x:c r="J26" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K26" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L26" s="58" t="str">
+      <x:c r="K26" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="73" t="str">
         <x:v>saria</x:v>
       </x:c>
-      <x:c r="M26" s="58" t="str">
+      <x:c r="M26" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N26" s="57" t="n">
+      <x:c r="N26" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O26" s="57" t="n">
+      <x:c r="O26" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P26" s="59" t="n">
+      <x:c r="P26" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q26" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R26" s="58" t="str">
+      <x:c r="Q26" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R26" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="57" t="n">
+      <x:c r="A27" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B27" s="58" t="str">
+      <x:c r="B27" s="73" t="str">
         <x:v>mode1_stage2_opening</x:v>
       </x:c>
-      <x:c r="C27" s="57" t="n">
+      <x:c r="C27" s="72" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D27" s="58" t="str">
+      <x:c r="D27" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E27" s="58" t="str">
+      <x:c r="E27" s="73" t="str">
         <x:v>上一关的强化已经消散，但元素选择和新的构筑会再次回应。两个人守住三条路线。</x:v>
       </x:c>
-      <x:c r="F27" s="58" t="str">
+      <x:c r="F27" s="73" t="str">
         <x:v>saria-soft</x:v>
       </x:c>
-      <x:c r="G27" s="58" t="str">
+      <x:c r="G27" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H27" s="57" t="n">
+      <x:c r="H27" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I27" s="57" t="n">
+      <x:c r="I27" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J27" s="59" t="n">
+      <x:c r="J27" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K27" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L27" s="58" t="str">
+      <x:c r="K27" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M27" s="58" t="str">
+      <x:c r="M27" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N27" s="57" t="n">
+      <x:c r="N27" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O27" s="57" t="n">
+      <x:c r="O27" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P27" s="59" t="n">
+      <x:c r="P27" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q27" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R27" s="58" t="str">
+      <x:c r="Q27" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R27" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="57" t="n">
+      <x:c r="A28" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B28" s="58" t="str">
+      <x:c r="B28" s="73" t="str">
         <x:v>mode1_stage3_opening</x:v>
       </x:c>
-      <x:c r="C28" s="57" t="n">
+      <x:c r="C28" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D28" s="58" t="str">
+      <x:c r="D28" s="73" t="str">
         <x:v>芙宁娜</x:v>
       </x:c>
-      <x:c r="E28" s="58" t="str">
+      <x:c r="E28" s="73" t="str">
         <x:v>第三道裂隙已经结晶化，路线正在上下错位。水域会替大家维持生命。</x:v>
       </x:c>
-      <x:c r="F28" s="58" t="str">
+      <x:c r="F28" s="73" t="str">
         <x:v>muelsyse</x:v>
       </x:c>
-      <x:c r="G28" s="58" t="str">
+      <x:c r="G28" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H28" s="57" t="n">
+      <x:c r="H28" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I28" s="57" t="n">
+      <x:c r="I28" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J28" s="59" t="n">
+      <x:c r="J28" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K28" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L28" s="58" t="str">
+      <x:c r="K28" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M28" s="58" t="str">
+      <x:c r="M28" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N28" s="57" t="n">
+      <x:c r="N28" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O28" s="57" t="n">
+      <x:c r="O28" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P28" s="59" t="n">
+      <x:c r="P28" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q28" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R28" s="58" t="str">
+      <x:c r="Q28" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R28" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="57" t="n">
+      <x:c r="A29" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="58" t="str">
+      <x:c r="B29" s="73" t="str">
         <x:v>mode1_stage3_opening</x:v>
       </x:c>
-      <x:c r="C29" s="57" t="n">
+      <x:c r="C29" s="72" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D29" s="58" t="str">
+      <x:c r="D29" s="73" t="str">
         <x:v>宵宫</x:v>
       </x:c>
-      <x:c r="E29" s="58" t="str">
+      <x:c r="E29" s="73" t="str">
         <x:v>黑曜母巢会周期召来疾行兽，我负责清掉它的护卫。</x:v>
       </x:c>
-      <x:c r="F29" s="58" t="str">
+      <x:c r="F29" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="G29" s="58" t="str">
+      <x:c r="G29" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H29" s="57" t="n">
+      <x:c r="H29" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I29" s="57" t="n">
+      <x:c r="I29" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J29" s="59" t="n">
+      <x:c r="J29" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K29" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L29" s="58" t="str">
+      <x:c r="K29" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="73" t="str">
         <x:v>muelsyse</x:v>
       </x:c>
-      <x:c r="M29" s="58" t="str">
+      <x:c r="M29" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N29" s="57" t="n">
+      <x:c r="N29" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O29" s="57" t="n">
+      <x:c r="O29" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P29" s="59" t="n">
+      <x:c r="P29" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q29" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R29" s="58" t="str">
+      <x:c r="Q29" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R29" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="57" t="n">
+      <x:c r="A30" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B30" s="58" t="str">
+      <x:c r="B30" s="73" t="str">
         <x:v>mode1_stage3_opening</x:v>
       </x:c>
-      <x:c r="C30" s="57" t="n">
+      <x:c r="C30" s="72" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D30" s="58" t="str">
+      <x:c r="D30" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E30" s="58" t="str">
+      <x:c r="E30" s="73" t="str">
         <x:v>三人到齐。重新选择元素与构筑，把母巢留在这里。</x:v>
       </x:c>
-      <x:c r="F30" s="58" t="str">
+      <x:c r="F30" s="73" t="str">
         <x:v>saria-soft</x:v>
       </x:c>
-      <x:c r="G30" s="58" t="str">
+      <x:c r="G30" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H30" s="57" t="n">
+      <x:c r="H30" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I30" s="57" t="n">
+      <x:c r="I30" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J30" s="59" t="n">
+      <x:c r="J30" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K30" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L30" s="58" t="str">
+      <x:c r="K30" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="73" t="str">
         <x:v>muelsyse</x:v>
       </x:c>
-      <x:c r="M30" s="58" t="str">
+      <x:c r="M30" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N30" s="57" t="n">
+      <x:c r="N30" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O30" s="57" t="n">
+      <x:c r="O30" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P30" s="59" t="n">
+      <x:c r="P30" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q30" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R30" s="58" t="str">
+      <x:c r="Q30" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R30" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
-      <x:c r="A31" s="57" t="n">
+      <x:c r="A31" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B31" s="58" t="str">
+      <x:c r="B31" s="73" t="str">
         <x:v>mode1_final_won</x:v>
       </x:c>
-      <x:c r="C31" s="57" t="n">
+      <x:c r="C31" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D31" s="58" t="str">
+      <x:c r="D31" s="73" t="str">
         <x:v>芙宁娜</x:v>
       </x:c>
-      <x:c r="E31" s="58" t="str">
+      <x:c r="E31" s="73" t="str">
         <x:v>黑曜母巢停止活动，三道裂隙都已经安静下来。</x:v>
       </x:c>
-      <x:c r="F31" s="58" t="str">
+      <x:c r="F31" s="73" t="str">
         <x:v>muelsyse</x:v>
       </x:c>
-      <x:c r="G31" s="58" t="str">
+      <x:c r="G31" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H31" s="57" t="n">
+      <x:c r="H31" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I31" s="57" t="n">
+      <x:c r="I31" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J31" s="59" t="n">
+      <x:c r="J31" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K31" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L31" s="58" t="str">
+      <x:c r="K31" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="73" t="str">
         <x:v>saria</x:v>
       </x:c>
-      <x:c r="M31" s="58" t="str">
+      <x:c r="M31" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N31" s="57" t="n">
+      <x:c r="N31" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O31" s="57" t="n">
+      <x:c r="O31" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P31" s="59" t="n">
+      <x:c r="P31" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q31" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R31" s="58" t="str">
+      <x:c r="Q31" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R31" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
-      <x:c r="A32" s="57" t="n">
+      <x:c r="A32" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B32" s="58" t="str">
+      <x:c r="B32" s="73" t="str">
         <x:v>mode1_final_won</x:v>
       </x:c>
-      <x:c r="C32" s="57" t="n">
+      <x:c r="C32" s="72" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D32" s="58" t="str">
+      <x:c r="D32" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E32" s="58" t="str">
+      <x:c r="E32" s="73" t="str">
         <x:v>模式一的防线全部守住，水晶已经记录新的角色与卡牌。</x:v>
       </x:c>
-      <x:c r="F32" s="58" t="str">
+      <x:c r="F32" s="73" t="str">
         <x:v>saria-soft</x:v>
       </x:c>
-      <x:c r="G32" s="58" t="str">
+      <x:c r="G32" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H32" s="57" t="n">
+      <x:c r="H32" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I32" s="57" t="n">
+      <x:c r="I32" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J32" s="59" t="n">
+      <x:c r="J32" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K32" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L32" s="58" t="str">
+      <x:c r="K32" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="73" t="str">
         <x:v>muelsyse</x:v>
       </x:c>
-      <x:c r="M32" s="58" t="str">
+      <x:c r="M32" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N32" s="57" t="n">
+      <x:c r="N32" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O32" s="57" t="n">
+      <x:c r="O32" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P32" s="59" t="n">
+      <x:c r="P32" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q32" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R32" s="58" t="str">
+      <x:c r="Q32" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R32" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
-      <x:c r="A33" s="57" t="n">
+      <x:c r="A33" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B33" s="58" t="str">
+      <x:c r="B33" s="73" t="str">
         <x:v>mode1_lost</x:v>
       </x:c>
-      <x:c r="C33" s="57" t="n">
+      <x:c r="C33" s="72" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D33" s="58" t="str">
+      <x:c r="D33" s="73" t="str">
         <x:v>旅行者</x:v>
       </x:c>
-      <x:c r="E33" s="58" t="str">
+      <x:c r="E33" s="73" t="str">
         <x:v>水晶破碎前保住了核心记录。重来一次，这次把弹道铺满整条路线。</x:v>
       </x:c>
-      <x:c r="F33" s="58" t="str">
+      <x:c r="F33" s="73" t="str">
         <x:v>saria</x:v>
       </x:c>
-      <x:c r="G33" s="58" t="str">
+      <x:c r="G33" s="73" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="H33" s="57" t="n">
+      <x:c r="H33" s="72" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="I33" s="57" t="n">
+      <x:c r="I33" s="72" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J33" s="59" t="n">
+      <x:c r="J33" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K33" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L33" s="58" t="str">
+      <x:c r="K33" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="73" t="str">
         <x:v>jessica</x:v>
       </x:c>
-      <x:c r="M33" s="58" t="str">
+      <x:c r="M33" s="73" t="str">
         <x:v>right</x:v>
       </x:c>
-      <x:c r="N33" s="57" t="n">
+      <x:c r="N33" s="72" t="n">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="O33" s="57" t="n">
+      <x:c r="O33" s="72" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="P33" s="59" t="n">
+      <x:c r="P33" s="74" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q33" s="57" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R33" s="58" t="str">
+      <x:c r="Q33" s="72" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R33" s="73" t="str">
         <x:v>main</x:v>
       </x:c>
     </x:row>
@@ -13114,6 +13149,406 @@
       <x:c r="P564" s="68"/>
       <x:c r="Q564" s="68"/>
       <x:c r="R564" s="69"/>
+    </x:row>
+    <x:row r="565">
+      <x:c r="A565" s="76"/>
+      <x:c r="B565" s="77"/>
+      <x:c r="C565" s="77"/>
+      <x:c r="D565" s="77"/>
+      <x:c r="E565" s="77"/>
+      <x:c r="F565" s="77"/>
+      <x:c r="G565" s="77"/>
+      <x:c r="H565" s="77"/>
+      <x:c r="I565" s="77"/>
+      <x:c r="J565" s="77"/>
+      <x:c r="K565" s="77"/>
+      <x:c r="L565" s="77"/>
+      <x:c r="M565" s="77"/>
+      <x:c r="N565" s="77"/>
+      <x:c r="O565" s="77"/>
+      <x:c r="P565" s="77"/>
+      <x:c r="Q565" s="77"/>
+      <x:c r="R565" s="78"/>
+    </x:row>
+    <x:row r="566">
+      <x:c r="A566" s="79"/>
+      <x:c r="B566" s="80"/>
+      <x:c r="C566" s="80"/>
+      <x:c r="D566" s="80"/>
+      <x:c r="E566" s="80"/>
+      <x:c r="F566" s="80"/>
+      <x:c r="G566" s="80"/>
+      <x:c r="H566" s="80"/>
+      <x:c r="I566" s="80"/>
+      <x:c r="J566" s="80"/>
+      <x:c r="K566" s="80"/>
+      <x:c r="L566" s="80"/>
+      <x:c r="M566" s="80"/>
+      <x:c r="N566" s="80"/>
+      <x:c r="O566" s="80"/>
+      <x:c r="P566" s="80"/>
+      <x:c r="Q566" s="80"/>
+      <x:c r="R566" s="81"/>
+    </x:row>
+    <x:row r="567">
+      <x:c r="A567" s="79"/>
+      <x:c r="B567" s="80"/>
+      <x:c r="C567" s="80"/>
+      <x:c r="D567" s="80"/>
+      <x:c r="E567" s="80"/>
+      <x:c r="F567" s="80"/>
+      <x:c r="G567" s="80"/>
+      <x:c r="H567" s="80"/>
+      <x:c r="I567" s="80"/>
+      <x:c r="J567" s="80"/>
+      <x:c r="K567" s="80"/>
+      <x:c r="L567" s="80"/>
+      <x:c r="M567" s="80"/>
+      <x:c r="N567" s="80"/>
+      <x:c r="O567" s="80"/>
+      <x:c r="P567" s="80"/>
+      <x:c r="Q567" s="80"/>
+      <x:c r="R567" s="81"/>
+    </x:row>
+    <x:row r="568">
+      <x:c r="A568" s="79"/>
+      <x:c r="B568" s="80"/>
+      <x:c r="C568" s="80"/>
+      <x:c r="D568" s="80"/>
+      <x:c r="E568" s="80"/>
+      <x:c r="F568" s="80"/>
+      <x:c r="G568" s="80"/>
+      <x:c r="H568" s="80"/>
+      <x:c r="I568" s="80"/>
+      <x:c r="J568" s="80"/>
+      <x:c r="K568" s="80"/>
+      <x:c r="L568" s="80"/>
+      <x:c r="M568" s="80"/>
+      <x:c r="N568" s="80"/>
+      <x:c r="O568" s="80"/>
+      <x:c r="P568" s="80"/>
+      <x:c r="Q568" s="80"/>
+      <x:c r="R568" s="81"/>
+    </x:row>
+    <x:row r="569">
+      <x:c r="A569" s="79"/>
+      <x:c r="B569" s="80"/>
+      <x:c r="C569" s="80"/>
+      <x:c r="D569" s="80"/>
+      <x:c r="E569" s="80"/>
+      <x:c r="F569" s="80"/>
+      <x:c r="G569" s="80"/>
+      <x:c r="H569" s="80"/>
+      <x:c r="I569" s="80"/>
+      <x:c r="J569" s="80"/>
+      <x:c r="K569" s="80"/>
+      <x:c r="L569" s="80"/>
+      <x:c r="M569" s="80"/>
+      <x:c r="N569" s="80"/>
+      <x:c r="O569" s="80"/>
+      <x:c r="P569" s="80"/>
+      <x:c r="Q569" s="80"/>
+      <x:c r="R569" s="81"/>
+    </x:row>
+    <x:row r="570">
+      <x:c r="A570" s="79"/>
+      <x:c r="B570" s="80"/>
+      <x:c r="C570" s="80"/>
+      <x:c r="D570" s="80"/>
+      <x:c r="E570" s="80"/>
+      <x:c r="F570" s="80"/>
+      <x:c r="G570" s="80"/>
+      <x:c r="H570" s="80"/>
+      <x:c r="I570" s="80"/>
+      <x:c r="J570" s="80"/>
+      <x:c r="K570" s="80"/>
+      <x:c r="L570" s="80"/>
+      <x:c r="M570" s="80"/>
+      <x:c r="N570" s="80"/>
+      <x:c r="O570" s="80"/>
+      <x:c r="P570" s="80"/>
+      <x:c r="Q570" s="80"/>
+      <x:c r="R570" s="81"/>
+    </x:row>
+    <x:row r="571">
+      <x:c r="A571" s="79"/>
+      <x:c r="B571" s="80"/>
+      <x:c r="C571" s="80"/>
+      <x:c r="D571" s="80"/>
+      <x:c r="E571" s="80"/>
+      <x:c r="F571" s="80"/>
+      <x:c r="G571" s="80"/>
+      <x:c r="H571" s="80"/>
+      <x:c r="I571" s="80"/>
+      <x:c r="J571" s="80"/>
+      <x:c r="K571" s="80"/>
+      <x:c r="L571" s="80"/>
+      <x:c r="M571" s="80"/>
+      <x:c r="N571" s="80"/>
+      <x:c r="O571" s="80"/>
+      <x:c r="P571" s="80"/>
+      <x:c r="Q571" s="80"/>
+      <x:c r="R571" s="81"/>
+    </x:row>
+    <x:row r="572">
+      <x:c r="A572" s="79"/>
+      <x:c r="B572" s="80"/>
+      <x:c r="C572" s="80"/>
+      <x:c r="D572" s="80"/>
+      <x:c r="E572" s="80"/>
+      <x:c r="F572" s="80"/>
+      <x:c r="G572" s="80"/>
+      <x:c r="H572" s="80"/>
+      <x:c r="I572" s="80"/>
+      <x:c r="J572" s="80"/>
+      <x:c r="K572" s="80"/>
+      <x:c r="L572" s="80"/>
+      <x:c r="M572" s="80"/>
+      <x:c r="N572" s="80"/>
+      <x:c r="O572" s="80"/>
+      <x:c r="P572" s="80"/>
+      <x:c r="Q572" s="80"/>
+      <x:c r="R572" s="81"/>
+    </x:row>
+    <x:row r="573">
+      <x:c r="A573" s="79"/>
+      <x:c r="B573" s="80"/>
+      <x:c r="C573" s="80"/>
+      <x:c r="D573" s="80"/>
+      <x:c r="E573" s="80"/>
+      <x:c r="F573" s="80"/>
+      <x:c r="G573" s="80"/>
+      <x:c r="H573" s="80"/>
+      <x:c r="I573" s="80"/>
+      <x:c r="J573" s="80"/>
+      <x:c r="K573" s="80"/>
+      <x:c r="L573" s="80"/>
+      <x:c r="M573" s="80"/>
+      <x:c r="N573" s="80"/>
+      <x:c r="O573" s="80"/>
+      <x:c r="P573" s="80"/>
+      <x:c r="Q573" s="80"/>
+      <x:c r="R573" s="81"/>
+    </x:row>
+    <x:row r="574">
+      <x:c r="A574" s="79"/>
+      <x:c r="B574" s="80"/>
+      <x:c r="C574" s="80"/>
+      <x:c r="D574" s="80"/>
+      <x:c r="E574" s="80"/>
+      <x:c r="F574" s="80"/>
+      <x:c r="G574" s="80"/>
+      <x:c r="H574" s="80"/>
+      <x:c r="I574" s="80"/>
+      <x:c r="J574" s="80"/>
+      <x:c r="K574" s="80"/>
+      <x:c r="L574" s="80"/>
+      <x:c r="M574" s="80"/>
+      <x:c r="N574" s="80"/>
+      <x:c r="O574" s="80"/>
+      <x:c r="P574" s="80"/>
+      <x:c r="Q574" s="80"/>
+      <x:c r="R574" s="81"/>
+    </x:row>
+    <x:row r="575">
+      <x:c r="A575" s="79"/>
+      <x:c r="B575" s="80"/>
+      <x:c r="C575" s="80"/>
+      <x:c r="D575" s="80"/>
+      <x:c r="E575" s="80"/>
+      <x:c r="F575" s="80"/>
+      <x:c r="G575" s="80"/>
+      <x:c r="H575" s="80"/>
+      <x:c r="I575" s="80"/>
+      <x:c r="J575" s="80"/>
+      <x:c r="K575" s="80"/>
+      <x:c r="L575" s="80"/>
+      <x:c r="M575" s="80"/>
+      <x:c r="N575" s="80"/>
+      <x:c r="O575" s="80"/>
+      <x:c r="P575" s="80"/>
+      <x:c r="Q575" s="80"/>
+      <x:c r="R575" s="81"/>
+    </x:row>
+    <x:row r="576">
+      <x:c r="A576" s="79"/>
+      <x:c r="B576" s="80"/>
+      <x:c r="C576" s="80"/>
+      <x:c r="D576" s="80"/>
+      <x:c r="E576" s="80"/>
+      <x:c r="F576" s="80"/>
+      <x:c r="G576" s="80"/>
+      <x:c r="H576" s="80"/>
+      <x:c r="I576" s="80"/>
+      <x:c r="J576" s="80"/>
+      <x:c r="K576" s="80"/>
+      <x:c r="L576" s="80"/>
+      <x:c r="M576" s="80"/>
+      <x:c r="N576" s="80"/>
+      <x:c r="O576" s="80"/>
+      <x:c r="P576" s="80"/>
+      <x:c r="Q576" s="80"/>
+      <x:c r="R576" s="81"/>
+    </x:row>
+    <x:row r="577">
+      <x:c r="A577" s="79"/>
+      <x:c r="B577" s="80"/>
+      <x:c r="C577" s="80"/>
+      <x:c r="D577" s="80"/>
+      <x:c r="E577" s="80"/>
+      <x:c r="F577" s="80"/>
+      <x:c r="G577" s="80"/>
+      <x:c r="H577" s="80"/>
+      <x:c r="I577" s="80"/>
+      <x:c r="J577" s="80"/>
+      <x:c r="K577" s="80"/>
+      <x:c r="L577" s="80"/>
+      <x:c r="M577" s="80"/>
+      <x:c r="N577" s="80"/>
+      <x:c r="O577" s="80"/>
+      <x:c r="P577" s="80"/>
+      <x:c r="Q577" s="80"/>
+      <x:c r="R577" s="81"/>
+    </x:row>
+    <x:row r="578">
+      <x:c r="A578" s="79"/>
+      <x:c r="B578" s="80"/>
+      <x:c r="C578" s="80"/>
+      <x:c r="D578" s="80"/>
+      <x:c r="E578" s="80"/>
+      <x:c r="F578" s="80"/>
+      <x:c r="G578" s="80"/>
+      <x:c r="H578" s="80"/>
+      <x:c r="I578" s="80"/>
+      <x:c r="J578" s="80"/>
+      <x:c r="K578" s="80"/>
+      <x:c r="L578" s="80"/>
+      <x:c r="M578" s="80"/>
+      <x:c r="N578" s="80"/>
+      <x:c r="O578" s="80"/>
+      <x:c r="P578" s="80"/>
+      <x:c r="Q578" s="80"/>
+      <x:c r="R578" s="81"/>
+    </x:row>
+    <x:row r="579">
+      <x:c r="A579" s="79"/>
+      <x:c r="B579" s="80"/>
+      <x:c r="C579" s="80"/>
+      <x:c r="D579" s="80"/>
+      <x:c r="E579" s="80"/>
+      <x:c r="F579" s="80"/>
+      <x:c r="G579" s="80"/>
+      <x:c r="H579" s="80"/>
+      <x:c r="I579" s="80"/>
+      <x:c r="J579" s="80"/>
+      <x:c r="K579" s="80"/>
+      <x:c r="L579" s="80"/>
+      <x:c r="M579" s="80"/>
+      <x:c r="N579" s="80"/>
+      <x:c r="O579" s="80"/>
+      <x:c r="P579" s="80"/>
+      <x:c r="Q579" s="80"/>
+      <x:c r="R579" s="81"/>
+    </x:row>
+    <x:row r="580">
+      <x:c r="A580" s="79"/>
+      <x:c r="B580" s="80"/>
+      <x:c r="C580" s="80"/>
+      <x:c r="D580" s="80"/>
+      <x:c r="E580" s="80"/>
+      <x:c r="F580" s="80"/>
+      <x:c r="G580" s="80"/>
+      <x:c r="H580" s="80"/>
+      <x:c r="I580" s="80"/>
+      <x:c r="J580" s="80"/>
+      <x:c r="K580" s="80"/>
+      <x:c r="L580" s="80"/>
+      <x:c r="M580" s="80"/>
+      <x:c r="N580" s="80"/>
+      <x:c r="O580" s="80"/>
+      <x:c r="P580" s="80"/>
+      <x:c r="Q580" s="80"/>
+      <x:c r="R580" s="81"/>
+    </x:row>
+    <x:row r="581">
+      <x:c r="A581" s="79"/>
+      <x:c r="B581" s="80"/>
+      <x:c r="C581" s="80"/>
+      <x:c r="D581" s="80"/>
+      <x:c r="E581" s="80"/>
+      <x:c r="F581" s="80"/>
+      <x:c r="G581" s="80"/>
+      <x:c r="H581" s="80"/>
+      <x:c r="I581" s="80"/>
+      <x:c r="J581" s="80"/>
+      <x:c r="K581" s="80"/>
+      <x:c r="L581" s="80"/>
+      <x:c r="M581" s="80"/>
+      <x:c r="N581" s="80"/>
+      <x:c r="O581" s="80"/>
+      <x:c r="P581" s="80"/>
+      <x:c r="Q581" s="80"/>
+      <x:c r="R581" s="81"/>
+    </x:row>
+    <x:row r="582">
+      <x:c r="A582" s="79"/>
+      <x:c r="B582" s="80"/>
+      <x:c r="C582" s="80"/>
+      <x:c r="D582" s="80"/>
+      <x:c r="E582" s="80"/>
+      <x:c r="F582" s="80"/>
+      <x:c r="G582" s="80"/>
+      <x:c r="H582" s="80"/>
+      <x:c r="I582" s="80"/>
+      <x:c r="J582" s="80"/>
+      <x:c r="K582" s="80"/>
+      <x:c r="L582" s="80"/>
+      <x:c r="M582" s="80"/>
+      <x:c r="N582" s="80"/>
+      <x:c r="O582" s="80"/>
+      <x:c r="P582" s="80"/>
+      <x:c r="Q582" s="80"/>
+      <x:c r="R582" s="81"/>
+    </x:row>
+    <x:row r="583">
+      <x:c r="A583" s="79"/>
+      <x:c r="B583" s="80"/>
+      <x:c r="C583" s="80"/>
+      <x:c r="D583" s="80"/>
+      <x:c r="E583" s="80"/>
+      <x:c r="F583" s="80"/>
+      <x:c r="G583" s="80"/>
+      <x:c r="H583" s="80"/>
+      <x:c r="I583" s="80"/>
+      <x:c r="J583" s="80"/>
+      <x:c r="K583" s="80"/>
+      <x:c r="L583" s="80"/>
+      <x:c r="M583" s="80"/>
+      <x:c r="N583" s="80"/>
+      <x:c r="O583" s="80"/>
+      <x:c r="P583" s="80"/>
+      <x:c r="Q583" s="80"/>
+      <x:c r="R583" s="81"/>
+    </x:row>
+    <x:row r="584">
+      <x:c r="A584" s="82"/>
+      <x:c r="B584" s="83"/>
+      <x:c r="C584" s="83"/>
+      <x:c r="D584" s="83"/>
+      <x:c r="E584" s="83"/>
+      <x:c r="F584" s="83"/>
+      <x:c r="G584" s="83"/>
+      <x:c r="H584" s="83"/>
+      <x:c r="I584" s="83"/>
+      <x:c r="J584" s="83"/>
+      <x:c r="K584" s="83"/>
+      <x:c r="L584" s="83"/>
+      <x:c r="M584" s="83"/>
+      <x:c r="N584" s="83"/>
+      <x:c r="O584" s="83"/>
+      <x:c r="P584" s="83"/>
+      <x:c r="Q584" s="83"/>
+      <x:c r="R584" s="84"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="6">
@@ -13271,16 +13706,16 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="70" t="str">
+      <x:c r="A11" s="85" t="str">
         <x:v>ui.bg.archive</x:v>
       </x:c>
-      <x:c r="B11" s="70" t="str">
+      <x:c r="B11" s="85" t="str">
         <x:v>res://assets/helltaker/backgrounds/chapterBG0008.png</x:v>
       </x:c>
-      <x:c r="C11" s="70" t="str">
+      <x:c r="C11" s="85" t="str">
         <x:v>编队与图鉴背景</x:v>
       </x:c>
-      <x:c r="D11" s="70" t="str">
+      <x:c r="D11" s="85" t="str">
         <x:v>UI背景</x:v>
       </x:c>
     </x:row>
@@ -14893,10 +15328,10 @@
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="21" t="str">
-        <x:v>squad_button</x:v>
+        <x:v>stage_button</x:v>
       </x:c>
       <x:c r="B26" s="20" t="n">
-        <x:v>570</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="C26" s="20" t="n">
         <x:v>8</x:v>
@@ -14912,7 +15347,7 @@
         <x:v>stretch</x:v>
       </x:c>
       <x:c r="H26" s="19" t="str">
-        <x:v>编队  [F3]</x:v>
+        <x:v>关卡  [F4]</x:v>
       </x:c>
       <x:c r="I26" s="20" t="n">
         <x:v>14</x:v>
@@ -14930,7 +15365,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="20" t="str">
-        <x:v>战斗顶部编队入口</x:v>
+        <x:v>战斗顶部关卡入口</x:v>
       </x:c>
       <x:c r="O26" s="20" t="n">
         <x:v>1</x:v>
@@ -14938,29 +15373,29 @@
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="21" t="str">
-        <x:v>squad_background</x:v>
+        <x:v>squad_button</x:v>
       </x:c>
       <x:c r="B27" s="20" t="n">
-        <x:v>0</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="C27" s="20" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D27" s="20" t="n">
-        <x:v>1280</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="E27" s="20" t="n">
-        <x:v>720</x:v>
-      </x:c>
-      <x:c r="F27" s="19" t="str">
-        <x:v>ui.bg.archive</x:v>
-      </x:c>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str"/>
       <x:c r="G27" s="19" t="str">
         <x:v>stretch</x:v>
       </x:c>
-      <x:c r="H27" s="19" t="str"/>
+      <x:c r="H27" s="19" t="str">
+        <x:v>编队  [F3]</x:v>
+      </x:c>
       <x:c r="I27" s="20" t="n">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J27" s="20" t="n">
         <x:v>0</x:v>
@@ -14975,7 +15410,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="20" t="str">
-        <x:v>编队页背景</x:v>
+        <x:v>战斗顶部编队入口</x:v>
       </x:c>
       <x:c r="O27" s="20" t="n">
         <x:v>1</x:v>
@@ -14983,21 +15418,23 @@
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
       <x:c r="A28" s="21" t="str">
-        <x:v>squad_frame</x:v>
+        <x:v>squad_background</x:v>
       </x:c>
       <x:c r="B28" s="20" t="n">
-        <x:v>72</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C28" s="20" t="n">
-        <x:v>42</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D28" s="20" t="n">
-        <x:v>1136</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="E28" s="20" t="n">
-        <x:v>636</x:v>
-      </x:c>
-      <x:c r="F28" s="19" t="str"/>
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="F28" s="19" t="str">
+        <x:v>ui.bg.archive</x:v>
+      </x:c>
       <x:c r="G28" s="19" t="str">
         <x:v>stretch</x:v>
       </x:c>
@@ -15018,7 +15455,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="20" t="str">
-        <x:v>编队页主框</x:v>
+        <x:v>编队页背景</x:v>
       </x:c>
       <x:c r="O28" s="20" t="n">
         <x:v>1</x:v>
@@ -15026,19 +15463,19 @@
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
       <x:c r="A29" s="21" t="str">
-        <x:v>squad_title</x:v>
+        <x:v>squad_frame</x:v>
       </x:c>
       <x:c r="B29" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C29" s="20" t="n">
-        <x:v>50</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D29" s="20" t="n">
-        <x:v>700</x:v>
+        <x:v>1136</x:v>
       </x:c>
       <x:c r="E29" s="20" t="n">
-        <x:v>42</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="F29" s="19" t="str"/>
       <x:c r="G29" s="19" t="str">
@@ -15046,7 +15483,7 @@
       </x:c>
       <x:c r="H29" s="19" t="str"/>
       <x:c r="I29" s="20" t="n">
-        <x:v>30</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J29" s="20" t="n">
         <x:v>0</x:v>
@@ -15061,7 +15498,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="20" t="str">
-        <x:v>下一关标题</x:v>
+        <x:v>编队页主框</x:v>
       </x:c>
       <x:c r="O29" s="20" t="n">
         <x:v>1</x:v>
@@ -15069,19 +15506,19 @@
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
       <x:c r="A30" s="21" t="str">
-        <x:v>squad_subtitle</x:v>
+        <x:v>squad_title</x:v>
       </x:c>
       <x:c r="B30" s="20" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="C30" s="20" t="n">
-        <x:v>94</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D30" s="20" t="n">
-        <x:v>900</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="E30" s="20" t="n">
-        <x:v>24</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F30" s="19" t="str"/>
       <x:c r="G30" s="19" t="str">
@@ -15089,7 +15526,7 @@
       </x:c>
       <x:c r="H30" s="19" t="str"/>
       <x:c r="I30" s="20" t="n">
-        <x:v>14</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="J30" s="20" t="n">
         <x:v>0</x:v>
@@ -15104,7 +15541,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="20" t="str">
-        <x:v>解锁提示</x:v>
+        <x:v>下一关标题</x:v>
       </x:c>
       <x:c r="O30" s="20" t="n">
         <x:v>1</x:v>
@@ -15112,29 +15549,27 @@
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
       <x:c r="A31" s="21" t="str">
-        <x:v>squad_confirm</x:v>
+        <x:v>squad_subtitle</x:v>
       </x:c>
       <x:c r="B31" s="20" t="n">
-        <x:v>308</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C31" s="20" t="n">
-        <x:v>500</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D31" s="20" t="n">
-        <x:v>520</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="E31" s="20" t="n">
-        <x:v>54</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F31" s="19" t="str"/>
       <x:c r="G31" s="19" t="str">
         <x:v>stretch</x:v>
       </x:c>
-      <x:c r="H31" s="19" t="str">
-        <x:v>确认编队并进入下一关   →</x:v>
-      </x:c>
+      <x:c r="H31" s="19" t="str"/>
       <x:c r="I31" s="20" t="n">
-        <x:v>18</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J31" s="20" t="n">
         <x:v>0</x:v>
@@ -15149,7 +15584,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="20" t="str">
-        <x:v>确认按钮</x:v>
+        <x:v>解锁提示</x:v>
       </x:c>
       <x:c r="O31" s="20" t="n">
         <x:v>1</x:v>
@@ -15157,27 +15592,29 @@
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
       <x:c r="A32" s="21" t="str">
-        <x:v>squad_character_1</x:v>
+        <x:v>squad_confirm</x:v>
       </x:c>
       <x:c r="B32" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="C32" s="20" t="n">
-        <x:v>142</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="D32" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="E32" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str"/>
       <x:c r="G32" s="19" t="str">
         <x:v>stretch</x:v>
       </x:c>
-      <x:c r="H32" s="19" t="str"/>
+      <x:c r="H32" s="19" t="str">
+        <x:v>确认编队并进入下一关   →</x:v>
+      </x:c>
       <x:c r="I32" s="20" t="n">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J32" s="20" t="n">
         <x:v>0</x:v>
@@ -15192,7 +15629,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="20" t="str">
-        <x:v>角色槽位 1</x:v>
+        <x:v>确认按钮</x:v>
       </x:c>
       <x:c r="O32" s="20" t="n">
         <x:v>1</x:v>
@@ -15200,10 +15637,10 @@
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
       <x:c r="A33" s="21" t="str">
-        <x:v>squad_character_2</x:v>
+        <x:v>squad_character_1</x:v>
       </x:c>
       <x:c r="B33" s="20" t="n">
-        <x:v>304</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C33" s="20" t="n">
         <x:v>142</x:v>
@@ -15235,7 +15672,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="20" t="str">
-        <x:v>角色槽位 2</x:v>
+        <x:v>角色槽位 1</x:v>
       </x:c>
       <x:c r="O33" s="20" t="n">
         <x:v>1</x:v>
@@ -15243,10 +15680,10 @@
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
       <x:c r="A34" s="21" t="str">
-        <x:v>squad_character_3</x:v>
+        <x:v>squad_character_2</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>572</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C34" s="20" t="n">
         <x:v>142</x:v>
@@ -15278,7 +15715,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="20" t="str">
-        <x:v>角色槽位 3</x:v>
+        <x:v>角色槽位 2</x:v>
       </x:c>
       <x:c r="O34" s="20" t="n">
         <x:v>1</x:v>
@@ -15286,10 +15723,10 @@
     </x:row>
     <x:row r="35" ht="30" customHeight="1">
       <x:c r="A35" s="21" t="str">
-        <x:v>squad_character_4</x:v>
+        <x:v>squad_character_3</x:v>
       </x:c>
       <x:c r="B35" s="20" t="n">
-        <x:v>840</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="C35" s="20" t="n">
         <x:v>142</x:v>
@@ -15321,7 +15758,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N35" s="20" t="str">
-        <x:v>角色槽位 4</x:v>
+        <x:v>角色槽位 3</x:v>
       </x:c>
       <x:c r="O35" s="20" t="n">
         <x:v>1</x:v>
@@ -15329,13 +15766,13 @@
     </x:row>
     <x:row r="36" ht="30" customHeight="1">
       <x:c r="A36" s="21" t="str">
-        <x:v>squad_character_5</x:v>
+        <x:v>squad_character_4</x:v>
       </x:c>
       <x:c r="B36" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="C36" s="20" t="n">
-        <x:v>298</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D36" s="20" t="n">
         <x:v>250</x:v>
@@ -15364,7 +15801,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N36" s="20" t="str">
-        <x:v>角色槽位 5</x:v>
+        <x:v>角色槽位 4</x:v>
       </x:c>
       <x:c r="O36" s="20" t="n">
         <x:v>1</x:v>
@@ -15372,10 +15809,10 @@
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
       <x:c r="A37" s="21" t="str">
-        <x:v>squad_character_6</x:v>
+        <x:v>squad_character_5</x:v>
       </x:c>
       <x:c r="B37" s="20" t="n">
-        <x:v>304</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
         <x:v>298</x:v>
@@ -15407,7 +15844,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="20" t="str">
-        <x:v>角色槽位 6</x:v>
+        <x:v>角色槽位 5</x:v>
       </x:c>
       <x:c r="O37" s="20" t="n">
         <x:v>1</x:v>
@@ -15415,10 +15852,10 @@
     </x:row>
     <x:row r="38" ht="30" customHeight="1">
       <x:c r="A38" s="21" t="str">
-        <x:v>squad_character_7</x:v>
+        <x:v>squad_character_6</x:v>
       </x:c>
       <x:c r="B38" s="20" t="n">
-        <x:v>572</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C38" s="20" t="n">
         <x:v>298</x:v>
@@ -15450,7 +15887,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N38" s="20" t="str">
-        <x:v>角色槽位 7</x:v>
+        <x:v>角色槽位 6</x:v>
       </x:c>
       <x:c r="O38" s="20" t="n">
         <x:v>1</x:v>
@@ -15458,10 +15895,10 @@
     </x:row>
     <x:row r="39" ht="30" customHeight="1">
       <x:c r="A39" s="21" t="str">
-        <x:v>squad_character_8</x:v>
+        <x:v>squad_character_7</x:v>
       </x:c>
       <x:c r="B39" s="20" t="n">
-        <x:v>840</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="C39" s="20" t="n">
         <x:v>298</x:v>
@@ -15493,130 +15930,314 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N39" s="20" t="str">
-        <x:v>角色槽位 8</x:v>
+        <x:v>角色槽位 7</x:v>
       </x:c>
       <x:c r="O39" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="30" customHeight="1">
-      <x:c r="A40" s="12"/>
-      <x:c r="B40" s="14"/>
-      <x:c r="C40" s="14"/>
-      <x:c r="D40" s="14"/>
-      <x:c r="E40" s="14"/>
-      <x:c r="F40" s="12"/>
-      <x:c r="G40" s="12"/>
-      <x:c r="H40" s="13"/>
-      <x:c r="I40" s="14"/>
-      <x:c r="J40" s="14"/>
-      <x:c r="K40" s="14"/>
-      <x:c r="L40" s="14"/>
-      <x:c r="M40" s="14"/>
-      <x:c r="N40" s="13"/>
-      <x:c r="O40" s="14"/>
+      <x:c r="A40" s="21" t="str">
+        <x:v>squad_character_8</x:v>
+      </x:c>
+      <x:c r="B40" s="20" t="n">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="C40" s="20" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D40" s="20" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E40" s="20" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F40" s="19" t="str"/>
+      <x:c r="G40" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H40" s="19" t="str"/>
+      <x:c r="I40" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K40" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L40" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M40" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="20" t="str">
+        <x:v>角色槽位 8</x:v>
+      </x:c>
+      <x:c r="O40" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="30" customHeight="1">
-      <x:c r="A41" s="12"/>
-      <x:c r="B41" s="14"/>
-      <x:c r="C41" s="14"/>
-      <x:c r="D41" s="14"/>
-      <x:c r="E41" s="14"/>
-      <x:c r="F41" s="12"/>
-      <x:c r="G41" s="12"/>
-      <x:c r="H41" s="13"/>
-      <x:c r="I41" s="14"/>
-      <x:c r="J41" s="14"/>
-      <x:c r="K41" s="14"/>
-      <x:c r="L41" s="14"/>
-      <x:c r="M41" s="14"/>
-      <x:c r="N41" s="13"/>
-      <x:c r="O41" s="14"/>
+      <x:c r="A41" s="21" t="str">
+        <x:v>stage_background</x:v>
+      </x:c>
+      <x:c r="B41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="20" t="n">
+        <x:v>1280</x:v>
+      </x:c>
+      <x:c r="E41" s="20" t="n">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="F41" s="19" t="str"/>
+      <x:c r="G41" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H41" s="19" t="str"/>
+      <x:c r="I41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M41" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="20" t="str">
+        <x:v>关卡选择背景</x:v>
+      </x:c>
+      <x:c r="O41" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
-      <x:c r="A42" s="12"/>
-      <x:c r="B42" s="14"/>
-      <x:c r="C42" s="14"/>
-      <x:c r="D42" s="14"/>
-      <x:c r="E42" s="14"/>
-      <x:c r="F42" s="12"/>
-      <x:c r="G42" s="12"/>
-      <x:c r="H42" s="13"/>
-      <x:c r="I42" s="14"/>
-      <x:c r="J42" s="14"/>
-      <x:c r="K42" s="14"/>
-      <x:c r="L42" s="14"/>
-      <x:c r="M42" s="14"/>
-      <x:c r="N42" s="13"/>
-      <x:c r="O42" s="14"/>
+      <x:c r="A42" s="21" t="str">
+        <x:v>stage_frame</x:v>
+      </x:c>
+      <x:c r="B42" s="20" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C42" s="20" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D42" s="20" t="n">
+        <x:v>1136</x:v>
+      </x:c>
+      <x:c r="E42" s="20" t="n">
+        <x:v>592</x:v>
+      </x:c>
+      <x:c r="F42" s="19" t="str"/>
+      <x:c r="G42" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H42" s="19" t="str"/>
+      <x:c r="I42" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K42" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L42" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M42" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="20" t="str">
+        <x:v>关卡选择主框</x:v>
+      </x:c>
+      <x:c r="O42" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="30" customHeight="1">
-      <x:c r="A43" s="12"/>
-      <x:c r="B43" s="14"/>
-      <x:c r="C43" s="14"/>
-      <x:c r="D43" s="14"/>
-      <x:c r="E43" s="14"/>
-      <x:c r="F43" s="12"/>
-      <x:c r="G43" s="12"/>
-      <x:c r="H43" s="13"/>
-      <x:c r="I43" s="14"/>
-      <x:c r="J43" s="14"/>
-      <x:c r="K43" s="14"/>
-      <x:c r="L43" s="14"/>
-      <x:c r="M43" s="14"/>
-      <x:c r="N43" s="13"/>
-      <x:c r="O43" s="14"/>
+      <x:c r="A43" s="21" t="str">
+        <x:v>stage_title</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C43" s="20" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D43" s="20" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="E43" s="20" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F43" s="19" t="str"/>
+      <x:c r="G43" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H43" s="19" t="str">
+        <x:v>选择作战区域</x:v>
+      </x:c>
+      <x:c r="I43" s="20" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J43" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K43" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L43" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M43" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="20" t="str">
+        <x:v>关卡选择标题</x:v>
+      </x:c>
+      <x:c r="O43" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="30" customHeight="1">
-      <x:c r="A44" s="12"/>
-      <x:c r="B44" s="14"/>
-      <x:c r="C44" s="14"/>
-      <x:c r="D44" s="14"/>
-      <x:c r="E44" s="14"/>
-      <x:c r="F44" s="12"/>
-      <x:c r="G44" s="12"/>
-      <x:c r="H44" s="13"/>
-      <x:c r="I44" s="14"/>
-      <x:c r="J44" s="14"/>
-      <x:c r="K44" s="14"/>
-      <x:c r="L44" s="14"/>
-      <x:c r="M44" s="14"/>
-      <x:c r="N44" s="13"/>
-      <x:c r="O44" s="14"/>
+      <x:c r="A44" s="21" t="str">
+        <x:v>stage_card_1</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C44" s="20" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D44" s="20" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E44" s="20" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="F44" s="19" t="str"/>
+      <x:c r="G44" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H44" s="19" t="str"/>
+      <x:c r="I44" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J44" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K44" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L44" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M44" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="20" t="str">
+        <x:v>第一关卡片</x:v>
+      </x:c>
+      <x:c r="O44" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="30" customHeight="1">
-      <x:c r="A45" s="12"/>
-      <x:c r="B45" s="14"/>
-      <x:c r="C45" s="14"/>
-      <x:c r="D45" s="14"/>
-      <x:c r="E45" s="14"/>
-      <x:c r="F45" s="12"/>
-      <x:c r="G45" s="12"/>
-      <x:c r="H45" s="13"/>
-      <x:c r="I45" s="14"/>
-      <x:c r="J45" s="14"/>
-      <x:c r="K45" s="14"/>
-      <x:c r="L45" s="14"/>
-      <x:c r="M45" s="14"/>
-      <x:c r="N45" s="13"/>
-      <x:c r="O45" s="14"/>
+      <x:c r="A45" s="21" t="str">
+        <x:v>stage_card_2</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E45" s="20" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="F45" s="19" t="str"/>
+      <x:c r="G45" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H45" s="19" t="str"/>
+      <x:c r="I45" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J45" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K45" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L45" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M45" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="20" t="str">
+        <x:v>第二关卡片</x:v>
+      </x:c>
+      <x:c r="O45" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="30" customHeight="1">
-      <x:c r="A46" s="12"/>
-      <x:c r="B46" s="14"/>
-      <x:c r="C46" s="14"/>
-      <x:c r="D46" s="14"/>
-      <x:c r="E46" s="14"/>
-      <x:c r="F46" s="12"/>
-      <x:c r="G46" s="12"/>
-      <x:c r="H46" s="13"/>
-      <x:c r="I46" s="14"/>
-      <x:c r="J46" s="14"/>
-      <x:c r="K46" s="14"/>
-      <x:c r="L46" s="14"/>
-      <x:c r="M46" s="14"/>
-      <x:c r="N46" s="13"/>
-      <x:c r="O46" s="14"/>
+      <x:c r="A46" s="21" t="str">
+        <x:v>stage_card_3</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="n">
+        <x:v>746</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D46" s="20" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E46" s="20" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="F46" s="19" t="str"/>
+      <x:c r="G46" s="19" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H46" s="19" t="str"/>
+      <x:c r="I46" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J46" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K46" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L46" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M46" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N46" s="20" t="str">
+        <x:v>第三关卡片</x:v>
+      </x:c>
+      <x:c r="O46" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="30" customHeight="1">
       <x:c r="A47" s="12"/>

</xml_diff>

<commit_message>
feat: ship V19 visual combat and squad UI
</commit_message>
<xml_diff>
--- a/content/game_config.xlsx
+++ b/content/game_config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R15dbab3584914843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="Rf4dbd024d322463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="R34c7f9dc8ff244f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="Rc3e9e8734fcb492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R9f5af00b8c834c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="2" r:id="Rd967ed56d2b54023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片资源" sheetId="3" r:id="Rc7df99987db04c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="4" r:id="Rfa5dd6c6dd6348c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15466,16 +15466,16 @@
         <x:v>squad_frame</x:v>
       </x:c>
       <x:c r="B29" s="20" t="n">
-        <x:v>72</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C29" s="20" t="n">
-        <x:v>42</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D29" s="20" t="n">
-        <x:v>1136</x:v>
+        <x:v>1184</x:v>
       </x:c>
       <x:c r="E29" s="20" t="n">
-        <x:v>636</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="F29" s="19" t="str"/>
       <x:c r="G29" s="19" t="str">
@@ -15509,16 +15509,16 @@
         <x:v>squad_title</x:v>
       </x:c>
       <x:c r="B30" s="20" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C30" s="20" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D30" s="20" t="n">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="E30" s="20" t="n">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="C30" s="20" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D30" s="20" t="n">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="E30" s="20" t="n">
-        <x:v>42</x:v>
       </x:c>
       <x:c r="F30" s="19" t="str"/>
       <x:c r="G30" s="19" t="str">
@@ -15552,16 +15552,16 @@
         <x:v>squad_subtitle</x:v>
       </x:c>
       <x:c r="B31" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C31" s="20" t="n">
-        <x:v>94</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D31" s="20" t="n">
         <x:v>900</x:v>
       </x:c>
       <x:c r="E31" s="20" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F31" s="19" t="str"/>
       <x:c r="G31" s="19" t="str">
@@ -15595,16 +15595,16 @@
         <x:v>squad_confirm</x:v>
       </x:c>
       <x:c r="B32" s="20" t="n">
-        <x:v>308</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="C32" s="20" t="n">
-        <x:v>500</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="D32" s="20" t="n">
-        <x:v>520</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="E32" s="20" t="n">
-        <x:v>54</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str"/>
       <x:c r="G32" s="19" t="str">
@@ -15640,16 +15640,16 @@
         <x:v>squad_character_1</x:v>
       </x:c>
       <x:c r="B33" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C33" s="20" t="n">
-        <x:v>142</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D33" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E33" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F33" s="19" t="str"/>
       <x:c r="G33" s="19" t="str">
@@ -15683,16 +15683,16 @@
         <x:v>squad_character_2</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>304</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="C34" s="20" t="n">
-        <x:v>142</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D34" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E34" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F34" s="19" t="str"/>
       <x:c r="G34" s="19" t="str">
@@ -15726,16 +15726,16 @@
         <x:v>squad_character_3</x:v>
       </x:c>
       <x:c r="B35" s="20" t="n">
-        <x:v>572</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C35" s="20" t="n">
-        <x:v>142</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D35" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E35" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F35" s="19" t="str"/>
       <x:c r="G35" s="19" t="str">
@@ -15769,16 +15769,16 @@
         <x:v>squad_character_4</x:v>
       </x:c>
       <x:c r="B36" s="20" t="n">
-        <x:v>840</x:v>
+        <x:v>885</x:v>
       </x:c>
       <x:c r="C36" s="20" t="n">
-        <x:v>142</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D36" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E36" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F36" s="19" t="str"/>
       <x:c r="G36" s="19" t="str">
@@ -15812,16 +15812,16 @@
         <x:v>squad_character_5</x:v>
       </x:c>
       <x:c r="B37" s="20" t="n">
-        <x:v>36</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
-        <x:v>298</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="D37" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E37" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F37" s="19" t="str"/>
       <x:c r="G37" s="19" t="str">
@@ -15855,16 +15855,16 @@
         <x:v>squad_character_6</x:v>
       </x:c>
       <x:c r="B38" s="20" t="n">
-        <x:v>304</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="C38" s="20" t="n">
-        <x:v>298</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="D38" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E38" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F38" s="19" t="str"/>
       <x:c r="G38" s="19" t="str">
@@ -15898,16 +15898,16 @@
         <x:v>squad_character_7</x:v>
       </x:c>
       <x:c r="B39" s="20" t="n">
-        <x:v>572</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C39" s="20" t="n">
-        <x:v>298</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="D39" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E39" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F39" s="19" t="str"/>
       <x:c r="G39" s="19" t="str">
@@ -15941,16 +15941,16 @@
         <x:v>squad_character_8</x:v>
       </x:c>
       <x:c r="B40" s="20" t="n">
-        <x:v>840</x:v>
+        <x:v>885</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
-        <x:v>298</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="D40" s="20" t="n">
-        <x:v>250</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E40" s="20" t="n">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F40" s="19" t="str"/>
       <x:c r="G40" s="19" t="str">
@@ -16240,72 +16240,176 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="30" customHeight="1">
-      <x:c r="A47" s="12"/>
-      <x:c r="B47" s="14"/>
-      <x:c r="C47" s="14"/>
-      <x:c r="D47" s="14"/>
-      <x:c r="E47" s="14"/>
-      <x:c r="F47" s="12"/>
-      <x:c r="G47" s="12"/>
-      <x:c r="H47" s="13"/>
-      <x:c r="I47" s="14"/>
-      <x:c r="J47" s="14"/>
-      <x:c r="K47" s="14"/>
-      <x:c r="L47" s="14"/>
-      <x:c r="M47" s="14"/>
-      <x:c r="N47" s="13"/>
-      <x:c r="O47" s="14"/>
+      <x:c r="A47" s="12" t="str">
+        <x:v>squad_character_9</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="n">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str"/>
+      <x:c r="G47" s="12" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H47" s="13" t="str"/>
+      <x:c r="I47" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J47" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K47" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L47" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M47" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N47" s="13" t="str">
+        <x:v>角色槽位 9</x:v>
+      </x:c>
+      <x:c r="O47" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="30" customHeight="1">
-      <x:c r="A48" s="12"/>
-      <x:c r="B48" s="14"/>
-      <x:c r="C48" s="14"/>
-      <x:c r="D48" s="14"/>
-      <x:c r="E48" s="14"/>
-      <x:c r="F48" s="12"/>
-      <x:c r="G48" s="12"/>
-      <x:c r="H48" s="13"/>
-      <x:c r="I48" s="14"/>
-      <x:c r="J48" s="14"/>
-      <x:c r="K48" s="14"/>
-      <x:c r="L48" s="14"/>
-      <x:c r="M48" s="14"/>
-      <x:c r="N48" s="13"/>
-      <x:c r="O48" s="14"/>
+      <x:c r="A48" s="12" t="str">
+        <x:v>squad_character_10</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="n">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str"/>
+      <x:c r="G48" s="12" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H48" s="13" t="str"/>
+      <x:c r="I48" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J48" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K48" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L48" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M48" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N48" s="13" t="str">
+        <x:v>角色槽位 10</x:v>
+      </x:c>
+      <x:c r="O48" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="30" customHeight="1">
-      <x:c r="A49" s="12"/>
-      <x:c r="B49" s="14"/>
-      <x:c r="C49" s="14"/>
-      <x:c r="D49" s="14"/>
-      <x:c r="E49" s="14"/>
-      <x:c r="F49" s="12"/>
-      <x:c r="G49" s="12"/>
-      <x:c r="H49" s="13"/>
-      <x:c r="I49" s="14"/>
-      <x:c r="J49" s="14"/>
-      <x:c r="K49" s="14"/>
-      <x:c r="L49" s="14"/>
-      <x:c r="M49" s="14"/>
-      <x:c r="N49" s="13"/>
-      <x:c r="O49" s="14"/>
+      <x:c r="A49" s="12" t="str">
+        <x:v>squad_character_11</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="n">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str"/>
+      <x:c r="G49" s="12" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H49" s="13" t="str"/>
+      <x:c r="I49" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J49" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K49" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L49" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M49" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N49" s="13" t="str">
+        <x:v>角色槽位 11</x:v>
+      </x:c>
+      <x:c r="O49" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="30" customHeight="1">
-      <x:c r="A50" s="12"/>
-      <x:c r="B50" s="14"/>
-      <x:c r="C50" s="14"/>
-      <x:c r="D50" s="14"/>
-      <x:c r="E50" s="14"/>
-      <x:c r="F50" s="12"/>
-      <x:c r="G50" s="12"/>
-      <x:c r="H50" s="13"/>
-      <x:c r="I50" s="14"/>
-      <x:c r="J50" s="14"/>
-      <x:c r="K50" s="14"/>
-      <x:c r="L50" s="14"/>
-      <x:c r="M50" s="14"/>
-      <x:c r="N50" s="13"/>
-      <x:c r="O50" s="14"/>
+      <x:c r="A50" s="12" t="str">
+        <x:v>squad_character_12</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="n">
+        <x:v>885</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="n">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str"/>
+      <x:c r="G50" s="12" t="str">
+        <x:v>stretch</x:v>
+      </x:c>
+      <x:c r="H50" s="13" t="str"/>
+      <x:c r="I50" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J50" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K50" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L50" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M50" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N50" s="13" t="str">
+        <x:v>角色槽位 12</x:v>
+      </x:c>
+      <x:c r="O50" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="30" customHeight="1">
       <x:c r="A51" s="12"/>

</xml_diff>